<commit_message>
feat: IPO list as BSE table, calendar cells show company names directly
</commit_message>
<xml_diff>
--- a/docs/fakedata-reference.xlsx
+++ b/docs/fakedata-reference.xlsx
@@ -1,27 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="20394"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="14420"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wangqiong01\Desktop\个人文件\理财\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\songmuyi\Project\home-financial-assistant\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16714A5A-A64C-458A-8D5C-D8BC7E1BA7CF}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="25600" windowHeight="10280" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="25605" windowHeight="10275"/>
   </bookViews>
   <sheets>
     <sheet name="六月 (2)" sheetId="2" r:id="rId1"/>
     <sheet name="六月" sheetId="1" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="162913"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="48">
   <si>
     <t>参加活动</t>
   </si>
@@ -187,12 +186,16 @@
   <si>
     <t>SHT建行</t>
     <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>5月</t>
+    <phoneticPr fontId="12" type="noConversion"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="3">
     <numFmt numFmtId="176" formatCode="#,##0_ "/>
     <numFmt numFmtId="177" formatCode="0_ "/>
@@ -877,27 +880,27 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3FAE5DAB-3601-4168-B159-477C88B7F495}">
-  <dimension ref="A3:O82"/>
-  <sheetFormatPr defaultColWidth="10" defaultRowHeight="14" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A3:O80"/>
+  <sheetFormatPr defaultColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="12.1640625" customWidth="1"/>
-    <col min="2" max="2" width="5.1640625" style="11" customWidth="1"/>
-    <col min="3" max="3" width="14.6640625" customWidth="1"/>
+    <col min="1" max="1" width="12.125" customWidth="1"/>
+    <col min="2" max="2" width="5.125" style="11" customWidth="1"/>
+    <col min="3" max="3" width="14.625" customWidth="1"/>
     <col min="4" max="4" width="11.75" customWidth="1"/>
-    <col min="5" max="5" width="15.1640625" customWidth="1"/>
-    <col min="6" max="6" width="12.6640625" customWidth="1"/>
+    <col min="5" max="5" width="15.125" customWidth="1"/>
+    <col min="6" max="6" width="12.625" customWidth="1"/>
     <col min="7" max="7" width="13" customWidth="1"/>
-    <col min="8" max="9" width="12.83203125" customWidth="1"/>
-    <col min="10" max="10" width="15.1640625" customWidth="1"/>
-    <col min="11" max="11" width="12.83203125" customWidth="1"/>
+    <col min="8" max="9" width="12.875" customWidth="1"/>
+    <col min="10" max="10" width="15.125" customWidth="1"/>
+    <col min="11" max="11" width="12.875" customWidth="1"/>
     <col min="12" max="12" width="11.5" style="7" customWidth="1"/>
     <col min="13" max="13" width="24.25" style="8" customWidth="1"/>
-    <col min="14" max="14" width="10.58203125" style="8" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="10.58203125" customWidth="1"/>
+    <col min="14" max="14" width="10.625" style="8" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="10.625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:15" s="1" customFormat="1" ht="107.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:15" s="1" customFormat="1" ht="107.45" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B3" s="9"/>
       <c r="C3" s="10" t="s">
         <v>0</v>
@@ -918,7 +921,7 @@
       <c r="M3" s="30"/>
       <c r="N3" s="30"/>
     </row>
-    <row r="4" spans="1:15" s="2" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:15" s="2" customFormat="1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B4" s="11"/>
       <c r="C4" s="12" t="s">
         <v>31</v>
@@ -949,7 +952,7 @@
       </c>
       <c r="N4" s="32"/>
     </row>
-    <row r="5" spans="1:15" ht="17" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:15" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C5" s="13" t="s">
         <v>32</v>
       </c>
@@ -969,7 +972,7 @@
       <c r="J5" s="33"/>
       <c r="K5" s="33"/>
     </row>
-    <row r="6" spans="1:15" ht="17" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:15" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B6" s="15"/>
       <c r="C6" s="16" t="s">
         <v>4</v>
@@ -987,7 +990,7 @@
       <c r="J6" s="34"/>
       <c r="K6" s="34"/>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.2">
       <c r="B7" s="64" t="s">
         <v>28</v>
       </c>
@@ -1015,7 +1018,7 @@
         <v>7001241</v>
       </c>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.2">
       <c r="B8" s="64" t="s">
         <v>29</v>
       </c>
@@ -1041,7 +1044,7 @@
         <v>16710312</v>
       </c>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.2">
       <c r="B9" s="64" t="s">
         <v>8</v>
       </c>
@@ -1067,7 +1070,7 @@
         <v>18010379</v>
       </c>
     </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.2">
       <c r="B10" s="64" t="s">
         <v>9</v>
       </c>
@@ -1097,7 +1100,7 @@
       </c>
       <c r="O10" s="51"/>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.2">
       <c r="B11" s="64" t="s">
         <v>10</v>
       </c>
@@ -1123,7 +1126,7 @@
         <v>27650363</v>
       </c>
     </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:15" x14ac:dyDescent="0.2">
       <c r="B12" s="64" t="s">
         <v>11</v>
       </c>
@@ -1151,7 +1154,7 @@
       <c r="M12" s="59"/>
       <c r="O12" s="35"/>
     </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:15" x14ac:dyDescent="0.2">
       <c r="B13" s="64" t="s">
         <v>5</v>
       </c>
@@ -1178,7 +1181,7 @@
       </c>
       <c r="N13" s="62"/>
     </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:15" x14ac:dyDescent="0.2">
       <c r="B14" s="64" t="s">
         <v>6</v>
       </c>
@@ -1204,7 +1207,7 @@
         <v>10750529</v>
       </c>
     </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A15" s="57" t="s">
         <v>25</v>
       </c>
@@ -1233,7 +1236,7 @@
         <v>15750529</v>
       </c>
     </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:15" x14ac:dyDescent="0.2">
       <c r="B16" s="64" t="s">
         <v>8</v>
       </c>
@@ -1260,7 +1263,7 @@
         <v>18060433</v>
       </c>
     </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:12" x14ac:dyDescent="0.2">
       <c r="B17" s="64" t="s">
         <v>9</v>
       </c>
@@ -1284,7 +1287,7 @@
         <v>7008404</v>
       </c>
     </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:12" x14ac:dyDescent="0.2">
       <c r="B18" s="64" t="s">
         <v>10</v>
       </c>
@@ -1308,7 +1311,7 @@
         <v>17478230</v>
       </c>
     </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:12" x14ac:dyDescent="0.2">
       <c r="B19" s="64" t="s">
         <v>11</v>
       </c>
@@ -1332,7 +1335,7 @@
         <v>17489277</v>
       </c>
     </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A20" s="19"/>
       <c r="B20" s="64" t="s">
         <v>5</v>
@@ -1357,7 +1360,7 @@
         <v>17489277</v>
       </c>
     </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A21" s="19"/>
       <c r="B21" s="64" t="s">
         <v>6</v>
@@ -1384,7 +1387,7 @@
         <v>13319277</v>
       </c>
     </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A22" s="19"/>
       <c r="B22" s="64" t="s">
         <v>7</v>
@@ -1409,7 +1412,7 @@
         <v>11179277</v>
       </c>
     </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A23" s="19"/>
       <c r="B23" s="64" t="s">
         <v>8</v>
@@ -1438,7 +1441,7 @@
         <v>7119277</v>
       </c>
     </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A24" s="19"/>
       <c r="B24" s="64" t="s">
         <v>9</v>
@@ -1465,7 +1468,7 @@
         <v>17589277</v>
       </c>
     </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A25" s="19"/>
       <c r="B25" s="64" t="s">
         <v>10</v>
@@ -1492,7 +1495,7 @@
         <v>17589277</v>
       </c>
     </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A26" s="19"/>
       <c r="B26" s="64" t="s">
         <v>11</v>
@@ -1519,7 +1522,7 @@
         <v>17589277</v>
       </c>
     </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A27" s="19"/>
       <c r="B27" s="64" t="s">
         <v>5</v>
@@ -1546,7 +1549,7 @@
         <v>17589277</v>
       </c>
     </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A28" s="19"/>
       <c r="B28" s="64" t="s">
         <v>6</v>
@@ -1573,7 +1576,7 @@
         <v>7019277</v>
       </c>
     </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A29" s="19"/>
       <c r="B29" s="64" t="s">
         <v>7</v>
@@ -1602,7 +1605,7 @@
         <v>18719277</v>
       </c>
     </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A30" s="19"/>
       <c r="B30" s="64" t="s">
         <v>8</v>
@@ -1629,7 +1632,7 @@
         <v>7019277</v>
       </c>
     </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:12" x14ac:dyDescent="0.2">
       <c r="B31" s="64" t="s">
         <v>9</v>
       </c>
@@ -1653,7 +1656,7 @@
         <v>20219277</v>
       </c>
     </row>
-    <row r="32" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:12" x14ac:dyDescent="0.2">
       <c r="B32" s="64" t="s">
         <v>10</v>
       </c>
@@ -1679,7 +1682,7 @@
         <v>17609277</v>
       </c>
     </row>
-    <row r="33" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:14" x14ac:dyDescent="0.2">
       <c r="B33" s="64" t="s">
         <v>11</v>
       </c>
@@ -1706,7 +1709,7 @@
         <v>18199277</v>
       </c>
     </row>
-    <row r="34" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:14" x14ac:dyDescent="0.2">
       <c r="B34" s="64" t="s">
         <v>5</v>
       </c>
@@ -1732,7 +1735,7 @@
         <v>18379277</v>
       </c>
     </row>
-    <row r="35" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:14" x14ac:dyDescent="0.2">
       <c r="B35" s="64" t="s">
         <v>6</v>
       </c>
@@ -1758,7 +1761,7 @@
         <v>7019277</v>
       </c>
     </row>
-    <row r="36" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:14" x14ac:dyDescent="0.2">
       <c r="B36" s="64" t="s">
         <v>7</v>
       </c>
@@ -1782,7 +1785,7 @@
         <v>14789277</v>
       </c>
     </row>
-    <row r="37" spans="1:14" ht="17" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:14" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B37" s="15"/>
       <c r="C37" s="20" t="s">
         <v>12</v>
@@ -1811,7 +1814,7 @@
       </c>
       <c r="K37" s="38"/>
     </row>
-    <row r="38" spans="1:14" ht="17" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:14" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B38" s="15"/>
       <c r="C38" s="21" t="s">
         <v>13</v>
@@ -1840,7 +1843,7 @@
       </c>
       <c r="K38" s="40"/>
     </row>
-    <row r="39" spans="1:14" s="3" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:14" s="3" customFormat="1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B39" s="15"/>
       <c r="C39" s="22" t="s">
         <v>14</v>
@@ -1875,7 +1878,7 @@
       </c>
       <c r="N39" s="52"/>
     </row>
-    <row r="40" spans="1:14" s="4" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:14" s="4" customFormat="1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B40" s="11"/>
       <c r="C40" s="23" t="s">
         <v>15</v>
@@ -1894,7 +1897,7 @@
       <c r="M40" s="53"/>
       <c r="N40" s="53"/>
     </row>
-    <row r="41" spans="1:14" s="5" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:14" s="5" customFormat="1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B41" s="11"/>
       <c r="C41" s="10" t="s">
         <v>16</v>
@@ -1914,7 +1917,7 @@
       <c r="M41" s="54"/>
       <c r="N41" s="54"/>
     </row>
-    <row r="42" spans="1:14" ht="25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:14" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="F42" s="47"/>
       <c r="G42" s="47"/>
       <c r="H42" s="47"/>
@@ -1926,7 +1929,7 @@
         <v>193.6</v>
       </c>
     </row>
-    <row r="43" spans="1:14" ht="17" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:14" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="24"/>
       <c r="B43" s="25"/>
       <c r="C43" s="8" t="s">
@@ -1954,7 +1957,7 @@
       <c r="K43" s="49"/>
       <c r="M43" s="49"/>
     </row>
-    <row r="44" spans="1:14" ht="17" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:14" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C44" s="27" t="s">
         <v>19</v>
       </c>
@@ -1981,7 +1984,7 @@
       </c>
       <c r="K44" s="49"/>
     </row>
-    <row r="45" spans="1:14" ht="17" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:14" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C45" s="27"/>
       <c r="D45" s="28"/>
       <c r="E45" s="50" t="s">
@@ -2003,7 +2006,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:14" ht="17" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:14" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="E46" s="50" t="s">
         <v>22</v>
       </c>
@@ -2021,7 +2024,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:14" x14ac:dyDescent="0.2">
       <c r="E47" s="50" t="s">
         <v>26</v>
       </c>
@@ -2033,7 +2036,7 @@
       <c r="I47" s="47"/>
       <c r="J47" s="47"/>
     </row>
-    <row r="48" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:14" x14ac:dyDescent="0.2">
       <c r="C48" s="57" t="s">
         <v>35</v>
       </c>
@@ -2048,7 +2051,7 @@
       <c r="I48" s="47"/>
       <c r="J48" s="47"/>
     </row>
-    <row r="49" spans="3:10" x14ac:dyDescent="0.3">
+    <row r="49" spans="3:14" x14ac:dyDescent="0.2">
       <c r="C49" s="27" t="s">
         <v>36</v>
       </c>
@@ -2063,236 +2066,295 @@
       <c r="I49" s="47"/>
       <c r="J49" s="47"/>
     </row>
-    <row r="50" spans="3:10" x14ac:dyDescent="0.3">
+    <row r="50" spans="3:14" x14ac:dyDescent="0.2">
       <c r="F50" s="47"/>
       <c r="G50" s="47"/>
       <c r="H50" s="47"/>
       <c r="I50" s="47"/>
       <c r="J50" s="47"/>
     </row>
-    <row r="51" spans="3:10" x14ac:dyDescent="0.3">
+    <row r="51" spans="3:14" x14ac:dyDescent="0.2">
       <c r="F51" s="47"/>
       <c r="G51" s="47"/>
       <c r="H51" s="47"/>
       <c r="I51" s="47"/>
       <c r="J51" s="47"/>
     </row>
-    <row r="52" spans="3:10" x14ac:dyDescent="0.3">
+    <row r="52" spans="3:14" x14ac:dyDescent="0.2">
       <c r="F52" s="47"/>
       <c r="G52" s="47"/>
       <c r="H52" s="47"/>
       <c r="I52" s="47"/>
       <c r="J52" s="47"/>
     </row>
-    <row r="53" spans="3:10" x14ac:dyDescent="0.3">
+    <row r="53" spans="3:14" x14ac:dyDescent="0.2">
       <c r="F53" s="47"/>
       <c r="G53" s="47"/>
       <c r="H53" s="47"/>
       <c r="I53" s="47"/>
       <c r="J53" s="47"/>
     </row>
-    <row r="54" spans="3:10" x14ac:dyDescent="0.3">
+    <row r="54" spans="3:14" x14ac:dyDescent="0.2">
       <c r="F54" s="47"/>
       <c r="G54" s="47"/>
       <c r="H54" s="47"/>
       <c r="I54" s="47"/>
       <c r="J54" s="47"/>
     </row>
-    <row r="55" spans="3:10" x14ac:dyDescent="0.3">
+    <row r="55" spans="3:14" x14ac:dyDescent="0.2">
       <c r="F55" s="47"/>
       <c r="G55" s="47"/>
       <c r="H55" s="47"/>
       <c r="I55" s="47"/>
       <c r="J55" s="47"/>
     </row>
-    <row r="56" spans="3:10" x14ac:dyDescent="0.3">
+    <row r="56" spans="3:14" x14ac:dyDescent="0.2">
       <c r="F56" s="47"/>
       <c r="G56" s="47"/>
       <c r="H56" s="47"/>
       <c r="I56" s="47"/>
       <c r="J56" s="47"/>
     </row>
-    <row r="57" spans="3:10" x14ac:dyDescent="0.3">
+    <row r="57" spans="3:14" x14ac:dyDescent="0.2">
       <c r="F57" s="47"/>
       <c r="G57" s="47"/>
       <c r="H57" s="47"/>
       <c r="I57" s="47"/>
       <c r="J57" s="47"/>
     </row>
-    <row r="58" spans="3:10" x14ac:dyDescent="0.3">
+    <row r="58" spans="3:14" x14ac:dyDescent="0.2">
       <c r="F58" s="47"/>
       <c r="G58" s="47"/>
       <c r="H58" s="47"/>
       <c r="I58" s="47"/>
       <c r="J58" s="47"/>
     </row>
-    <row r="59" spans="3:10" x14ac:dyDescent="0.3">
+    <row r="59" spans="3:14" x14ac:dyDescent="0.2">
       <c r="F59" s="47"/>
       <c r="G59" s="47"/>
       <c r="H59" s="47"/>
       <c r="I59" s="47"/>
       <c r="J59" s="47"/>
     </row>
-    <row r="60" spans="3:10" x14ac:dyDescent="0.3">
+    <row r="60" spans="3:14" x14ac:dyDescent="0.2">
       <c r="F60" s="47"/>
       <c r="G60" s="47"/>
       <c r="H60" s="47"/>
       <c r="I60" s="47"/>
       <c r="J60" s="47"/>
     </row>
-    <row r="61" spans="3:10" x14ac:dyDescent="0.3">
+    <row r="61" spans="3:14" x14ac:dyDescent="0.2">
+      <c r="D61" s="47"/>
+      <c r="E61" s="47"/>
       <c r="F61" s="47"/>
       <c r="G61" s="47"/>
       <c r="H61" s="47"/>
-      <c r="I61" s="47"/>
-      <c r="J61" s="47"/>
-    </row>
-    <row r="62" spans="3:10" x14ac:dyDescent="0.3">
-      <c r="F62" s="47"/>
-      <c r="G62" s="47"/>
-      <c r="H62" s="47"/>
-      <c r="I62" s="47"/>
-      <c r="J62" s="47"/>
-    </row>
-    <row r="63" spans="3:10" x14ac:dyDescent="0.3">
-      <c r="F63" s="47"/>
-      <c r="G63" s="47"/>
-      <c r="H63" s="47"/>
-      <c r="I63" s="47"/>
-      <c r="J63" s="47"/>
-    </row>
-    <row r="64" spans="3:10" x14ac:dyDescent="0.3">
-      <c r="F64" s="47"/>
-      <c r="G64" s="47"/>
-      <c r="H64" s="47"/>
-      <c r="I64" s="47"/>
-      <c r="J64" s="47"/>
-    </row>
-    <row r="65" spans="6:10" x14ac:dyDescent="0.3">
-      <c r="F65" s="47"/>
-      <c r="G65" s="47"/>
-      <c r="H65" s="47"/>
-      <c r="I65" s="47"/>
-      <c r="J65" s="47"/>
-    </row>
-    <row r="66" spans="6:10" x14ac:dyDescent="0.3">
+      <c r="J61" s="7"/>
+      <c r="K61" s="8"/>
+      <c r="L61" s="8"/>
+      <c r="M61"/>
+      <c r="N61"/>
+    </row>
+    <row r="62" spans="3:14" ht="15.75" x14ac:dyDescent="0.2">
+      <c r="C62" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="D62" s="31" t="s">
+        <v>30</v>
+      </c>
+      <c r="E62" s="31" t="s">
+        <v>33</v>
+      </c>
+      <c r="F62" s="31" t="s">
+        <v>38</v>
+      </c>
+      <c r="G62" s="31" t="s">
+        <v>46</v>
+      </c>
+      <c r="H62" s="31" t="s">
+        <v>2</v>
+      </c>
+      <c r="I62" s="7"/>
+      <c r="J62" s="8"/>
+      <c r="K62" s="8"/>
+      <c r="L62"/>
+      <c r="M62"/>
+      <c r="N62"/>
+    </row>
+    <row r="63" spans="3:14" x14ac:dyDescent="0.2">
+      <c r="C63" s="18">
+        <v>46145</v>
+      </c>
+      <c r="D63" s="36"/>
+      <c r="E63" s="36">
+        <v>15000000</v>
+      </c>
+      <c r="F63" s="36"/>
+      <c r="G63" s="36"/>
+      <c r="H63" s="35" t="s">
+        <v>37</v>
+      </c>
+      <c r="I63" s="7"/>
+      <c r="J63" s="8"/>
+      <c r="K63" s="8"/>
+      <c r="L63"/>
+      <c r="M63"/>
+      <c r="N63"/>
+    </row>
+    <row r="64" spans="3:14" x14ac:dyDescent="0.2">
+      <c r="C64" s="18">
+        <v>46146</v>
+      </c>
+      <c r="D64" s="36">
+        <v>55000</v>
+      </c>
+      <c r="E64" s="36">
+        <v>15000000</v>
+      </c>
+      <c r="F64" s="36"/>
+      <c r="G64" s="36"/>
+      <c r="H64" s="35"/>
+      <c r="I64" s="7"/>
+      <c r="J64" s="8"/>
+      <c r="K64" s="8"/>
+      <c r="L64"/>
+      <c r="M64"/>
+      <c r="N64"/>
+    </row>
+    <row r="65" spans="3:14" x14ac:dyDescent="0.2">
+      <c r="C65" s="18">
+        <v>46147</v>
+      </c>
+      <c r="D65" s="36">
+        <v>240000</v>
+      </c>
+      <c r="E65" s="36"/>
+      <c r="F65" s="36">
+        <v>10200000</v>
+      </c>
+      <c r="G65" s="36"/>
+      <c r="H65" s="35"/>
+      <c r="I65" s="7"/>
+      <c r="J65" s="8"/>
+      <c r="K65" s="8"/>
+      <c r="L65"/>
+      <c r="M65"/>
+      <c r="N65"/>
+    </row>
+    <row r="66" spans="3:14" x14ac:dyDescent="0.2">
+      <c r="D66" s="47"/>
+      <c r="E66" s="47"/>
       <c r="F66" s="47"/>
       <c r="G66" s="47"/>
       <c r="H66" s="47"/>
-      <c r="I66" s="47"/>
-      <c r="J66" s="47"/>
-    </row>
-    <row r="67" spans="6:10" x14ac:dyDescent="0.3">
+      <c r="J66" s="7"/>
+      <c r="K66" s="8"/>
+      <c r="L66" s="8"/>
+      <c r="M66"/>
+      <c r="N66"/>
+    </row>
+    <row r="67" spans="3:14" x14ac:dyDescent="0.2">
+      <c r="D67" s="47"/>
+      <c r="E67" s="47"/>
       <c r="F67" s="47"/>
       <c r="G67" s="47"/>
       <c r="H67" s="47"/>
-      <c r="I67" s="47"/>
-      <c r="J67" s="47"/>
-    </row>
-    <row r="68" spans="6:10" x14ac:dyDescent="0.3">
+      <c r="J67" s="7"/>
+      <c r="K67" s="8"/>
+      <c r="L67" s="8"/>
+      <c r="M67"/>
+      <c r="N67"/>
+    </row>
+    <row r="68" spans="3:14" x14ac:dyDescent="0.2">
       <c r="F68" s="47"/>
       <c r="G68" s="47"/>
       <c r="H68" s="47"/>
       <c r="I68" s="47"/>
       <c r="J68" s="47"/>
     </row>
-    <row r="69" spans="6:10" x14ac:dyDescent="0.3">
+    <row r="69" spans="3:14" x14ac:dyDescent="0.2">
       <c r="F69" s="47"/>
       <c r="G69" s="47"/>
       <c r="H69" s="47"/>
       <c r="I69" s="47"/>
       <c r="J69" s="47"/>
     </row>
-    <row r="70" spans="6:10" x14ac:dyDescent="0.3">
+    <row r="70" spans="3:14" x14ac:dyDescent="0.2">
       <c r="F70" s="47"/>
       <c r="G70" s="47"/>
       <c r="H70" s="47"/>
       <c r="I70" s="47"/>
       <c r="J70" s="47"/>
     </row>
-    <row r="71" spans="6:10" x14ac:dyDescent="0.3">
+    <row r="71" spans="3:14" x14ac:dyDescent="0.2">
       <c r="F71" s="47"/>
       <c r="G71" s="47"/>
       <c r="H71" s="47"/>
       <c r="I71" s="47"/>
       <c r="J71" s="47"/>
     </row>
-    <row r="72" spans="6:10" x14ac:dyDescent="0.3">
+    <row r="72" spans="3:14" x14ac:dyDescent="0.2">
       <c r="F72" s="47"/>
       <c r="G72" s="47"/>
       <c r="H72" s="47"/>
       <c r="I72" s="47"/>
       <c r="J72" s="47"/>
     </row>
-    <row r="73" spans="6:10" x14ac:dyDescent="0.3">
+    <row r="73" spans="3:14" x14ac:dyDescent="0.2">
       <c r="F73" s="47"/>
       <c r="G73" s="47"/>
       <c r="H73" s="47"/>
       <c r="I73" s="47"/>
       <c r="J73" s="47"/>
     </row>
-    <row r="74" spans="6:10" x14ac:dyDescent="0.3">
+    <row r="74" spans="3:14" x14ac:dyDescent="0.2">
       <c r="F74" s="47"/>
       <c r="G74" s="47"/>
       <c r="H74" s="47"/>
       <c r="I74" s="47"/>
       <c r="J74" s="47"/>
     </row>
-    <row r="75" spans="6:10" x14ac:dyDescent="0.3">
+    <row r="75" spans="3:14" x14ac:dyDescent="0.2">
       <c r="F75" s="47"/>
       <c r="G75" s="47"/>
       <c r="H75" s="47"/>
       <c r="I75" s="47"/>
       <c r="J75" s="47"/>
     </row>
-    <row r="76" spans="6:10" x14ac:dyDescent="0.3">
+    <row r="76" spans="3:14" x14ac:dyDescent="0.2">
       <c r="F76" s="47"/>
       <c r="G76" s="47"/>
       <c r="H76" s="47"/>
       <c r="I76" s="47"/>
       <c r="J76" s="47"/>
     </row>
-    <row r="77" spans="6:10" x14ac:dyDescent="0.3">
+    <row r="77" spans="3:14" x14ac:dyDescent="0.2">
       <c r="F77" s="47"/>
       <c r="G77" s="47"/>
       <c r="H77" s="47"/>
       <c r="I77" s="47"/>
       <c r="J77" s="47"/>
     </row>
-    <row r="78" spans="6:10" x14ac:dyDescent="0.3">
+    <row r="78" spans="3:14" x14ac:dyDescent="0.2">
       <c r="F78" s="47"/>
       <c r="G78" s="47"/>
       <c r="H78" s="47"/>
       <c r="I78" s="47"/>
       <c r="J78" s="47"/>
     </row>
-    <row r="79" spans="6:10" x14ac:dyDescent="0.3">
+    <row r="79" spans="3:14" x14ac:dyDescent="0.2">
       <c r="F79" s="47"/>
       <c r="G79" s="47"/>
       <c r="H79" s="47"/>
       <c r="I79" s="47"/>
       <c r="J79" s="47"/>
     </row>
-    <row r="80" spans="6:10" x14ac:dyDescent="0.3">
+    <row r="80" spans="3:14" x14ac:dyDescent="0.2">
       <c r="F80" s="47"/>
       <c r="G80" s="47"/>
       <c r="H80" s="47"/>
       <c r="I80" s="47"/>
       <c r="J80" s="47"/>
-    </row>
-    <row r="81" spans="6:10" x14ac:dyDescent="0.3">
-      <c r="F81" s="47"/>
-      <c r="G81" s="47"/>
-      <c r="H81" s="47"/>
-      <c r="I81" s="47"/>
-      <c r="J81" s="47"/>
-    </row>
-    <row r="82" spans="6:10" x14ac:dyDescent="0.3">
-      <c r="F82" s="47"/>
-      <c r="G82" s="47"/>
-      <c r="H82" s="47"/>
-      <c r="I82" s="47"/>
-      <c r="J82" s="47"/>
     </row>
   </sheetData>
   <phoneticPr fontId="7" type="noConversion"/>
@@ -2302,27 +2364,27 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A3:N82"/>
-  <sheetFormatPr defaultColWidth="10" defaultRowHeight="14" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="12.1640625" customWidth="1"/>
-    <col min="2" max="2" width="5.1640625" style="6" customWidth="1"/>
-    <col min="3" max="3" width="14.6640625" customWidth="1"/>
+    <col min="1" max="1" width="12.125" customWidth="1"/>
+    <col min="2" max="2" width="5.125" style="6" customWidth="1"/>
+    <col min="3" max="3" width="14.625" customWidth="1"/>
     <col min="4" max="4" width="11.75" customWidth="1"/>
-    <col min="5" max="5" width="15.1640625" customWidth="1"/>
-    <col min="6" max="6" width="12.6640625" customWidth="1"/>
+    <col min="5" max="5" width="15.125" customWidth="1"/>
+    <col min="6" max="6" width="12.625" customWidth="1"/>
     <col min="7" max="7" width="13" customWidth="1"/>
-    <col min="8" max="8" width="12.83203125" customWidth="1"/>
-    <col min="9" max="9" width="15.1640625" customWidth="1"/>
-    <col min="10" max="10" width="12.83203125" customWidth="1"/>
+    <col min="8" max="8" width="12.875" customWidth="1"/>
+    <col min="9" max="9" width="15.125" customWidth="1"/>
+    <col min="10" max="10" width="12.875" customWidth="1"/>
     <col min="11" max="11" width="11.5" style="7" customWidth="1"/>
     <col min="12" max="12" width="24.25" style="8" customWidth="1"/>
-    <col min="13" max="13" width="10.58203125" style="8" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="10.58203125" customWidth="1"/>
+    <col min="13" max="13" width="10.625" style="8" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="10.625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:14" s="1" customFormat="1" ht="107.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:14" s="1" customFormat="1" ht="107.45" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B3" s="9"/>
       <c r="C3" s="10" t="s">
         <v>0</v>
@@ -2342,7 +2404,7 @@
       <c r="L3" s="30"/>
       <c r="M3" s="30"/>
     </row>
-    <row r="4" spans="1:14" s="2" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:14" s="2" customFormat="1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B4" s="11"/>
       <c r="C4" s="12" t="s">
         <v>31</v>
@@ -2368,7 +2430,7 @@
       </c>
       <c r="M4" s="32"/>
     </row>
-    <row r="5" spans="1:14" ht="17" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:14" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C5" s="13" t="s">
         <v>32</v>
       </c>
@@ -2384,7 +2446,7 @@
       <c r="I5" s="33"/>
       <c r="J5" s="33"/>
     </row>
-    <row r="6" spans="1:14" ht="17" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:14" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B6" s="15"/>
       <c r="C6" s="16" t="s">
         <v>4</v>
@@ -2401,7 +2463,7 @@
       <c r="I6" s="34"/>
       <c r="J6" s="34"/>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.2">
       <c r="B7" s="64" t="s">
         <v>28</v>
       </c>
@@ -2426,7 +2488,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.2">
       <c r="B8" s="64" t="s">
         <v>29</v>
       </c>
@@ -2449,7 +2511,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.2">
       <c r="B9" s="64" t="s">
         <v>8</v>
       </c>
@@ -2474,7 +2536,7 @@
         <v>10800000</v>
       </c>
     </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.2">
       <c r="B10" s="64" t="s">
         <v>9</v>
       </c>
@@ -2499,7 +2561,7 @@
       <c r="L10" s="59"/>
       <c r="N10" s="51"/>
     </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.2">
       <c r="B11" s="64" t="s">
         <v>10</v>
       </c>
@@ -2522,7 +2584,7 @@
         <v>10350000</v>
       </c>
     </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.2">
       <c r="B12" s="64" t="s">
         <v>11</v>
       </c>
@@ -2547,7 +2609,7 @@
       <c r="L12" s="59"/>
       <c r="N12" s="35"/>
     </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.2">
       <c r="B13" s="64" t="s">
         <v>5</v>
       </c>
@@ -2571,7 +2633,7 @@
       </c>
       <c r="M13" s="62"/>
     </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.2">
       <c r="B14" s="64" t="s">
         <v>6</v>
       </c>
@@ -2592,7 +2654,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A15" s="57" t="s">
         <v>25</v>
       </c>
@@ -2616,7 +2678,7 @@
         <v>10350000</v>
       </c>
     </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:14" x14ac:dyDescent="0.2">
       <c r="B16" s="64" t="s">
         <v>8</v>
       </c>
@@ -2637,7 +2699,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B17" s="64" t="s">
         <v>9</v>
       </c>
@@ -2658,7 +2720,7 @@
         <v>10350000</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B18" s="64" t="s">
         <v>10</v>
       </c>
@@ -2679,7 +2741,7 @@
         <v>10350000</v>
       </c>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B19" s="64" t="s">
         <v>11</v>
       </c>
@@ -2700,7 +2762,7 @@
         <v>10350000</v>
       </c>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A20" s="19"/>
       <c r="B20" s="64" t="s">
         <v>5</v>
@@ -2722,7 +2784,7 @@
         <v>10350000</v>
       </c>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A21" s="19"/>
       <c r="B21" s="64" t="s">
         <v>6</v>
@@ -2744,7 +2806,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A22" s="19"/>
       <c r="B22" s="64" t="s">
         <v>7</v>
@@ -2766,7 +2828,7 @@
         <v>10350000</v>
       </c>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A23" s="19"/>
       <c r="B23" s="64" t="s">
         <v>8</v>
@@ -2788,7 +2850,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A24" s="19"/>
       <c r="B24" s="64" t="s">
         <v>9</v>
@@ -2810,7 +2872,7 @@
         <v>10350000</v>
       </c>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A25" s="19"/>
       <c r="B25" s="64" t="s">
         <v>10</v>
@@ -2832,7 +2894,7 @@
         <v>10350000</v>
       </c>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A26" s="19"/>
       <c r="B26" s="64" t="s">
         <v>11</v>
@@ -2854,7 +2916,7 @@
         <v>10350000</v>
       </c>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A27" s="19"/>
       <c r="B27" s="64" t="s">
         <v>5</v>
@@ -2876,7 +2938,7 @@
         <v>10350000</v>
       </c>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A28" s="19"/>
       <c r="B28" s="64" t="s">
         <v>6</v>
@@ -2898,7 +2960,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A29" s="19"/>
       <c r="B29" s="64" t="s">
         <v>7</v>
@@ -2920,7 +2982,7 @@
         <v>10350000</v>
       </c>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A30" s="19"/>
       <c r="B30" s="64" t="s">
         <v>8</v>
@@ -2942,7 +3004,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B31" s="64" t="s">
         <v>9</v>
       </c>
@@ -2963,7 +3025,7 @@
         <v>10350000</v>
       </c>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B32" s="64" t="s">
         <v>10</v>
       </c>
@@ -2984,7 +3046,7 @@
         <v>10350000</v>
       </c>
     </row>
-    <row r="33" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:13" x14ac:dyDescent="0.2">
       <c r="B33" s="64" t="s">
         <v>11</v>
       </c>
@@ -3005,7 +3067,7 @@
         <v>10350000</v>
       </c>
     </row>
-    <row r="34" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:13" x14ac:dyDescent="0.2">
       <c r="B34" s="64" t="s">
         <v>5</v>
       </c>
@@ -3026,7 +3088,7 @@
         <v>10350000</v>
       </c>
     </row>
-    <row r="35" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:13" x14ac:dyDescent="0.2">
       <c r="B35" s="64" t="s">
         <v>6</v>
       </c>
@@ -3047,7 +3109,7 @@
         <v>10350000</v>
       </c>
     </row>
-    <row r="36" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:13" x14ac:dyDescent="0.2">
       <c r="B36" s="64" t="s">
         <v>7</v>
       </c>
@@ -3068,7 +3130,7 @@
         <v>10350000</v>
       </c>
     </row>
-    <row r="37" spans="1:13" ht="17" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:13" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B37" s="15"/>
       <c r="C37" s="20" t="s">
         <v>12</v>
@@ -3093,7 +3155,7 @@
       </c>
       <c r="J37" s="38"/>
     </row>
-    <row r="38" spans="1:13" ht="17" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:13" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B38" s="15"/>
       <c r="C38" s="21" t="s">
         <v>13</v>
@@ -3118,7 +3180,7 @@
       </c>
       <c r="J38" s="40"/>
     </row>
-    <row r="39" spans="1:13" s="3" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:13" s="3" customFormat="1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B39" s="15"/>
       <c r="C39" s="22" t="s">
         <v>14</v>
@@ -3146,7 +3208,7 @@
       <c r="L39" s="52"/>
       <c r="M39" s="52"/>
     </row>
-    <row r="40" spans="1:13" s="4" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:13" s="4" customFormat="1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B40" s="11"/>
       <c r="C40" s="23" t="s">
         <v>15</v>
@@ -3164,7 +3226,7 @@
       <c r="L40" s="53"/>
       <c r="M40" s="53"/>
     </row>
-    <row r="41" spans="1:13" s="5" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:13" s="5" customFormat="1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B41" s="11"/>
       <c r="C41" s="10" t="s">
         <v>16</v>
@@ -3180,7 +3242,7 @@
       <c r="L41" s="54"/>
       <c r="M41" s="54"/>
     </row>
-    <row r="42" spans="1:13" ht="25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:13" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="F42" s="47"/>
       <c r="G42" s="47"/>
       <c r="H42" s="47"/>
@@ -3191,7 +3253,7 @@
         <v>193.6</v>
       </c>
     </row>
-    <row r="43" spans="1:13" ht="17" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:13" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="24"/>
       <c r="B43" s="25"/>
       <c r="C43" s="8" t="s">
@@ -3214,7 +3276,7 @@
       <c r="J43" s="49"/>
       <c r="L43" s="49"/>
     </row>
-    <row r="44" spans="1:13" ht="17" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:13" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C44" s="27" t="s">
         <v>19</v>
       </c>
@@ -3237,7 +3299,7 @@
       </c>
       <c r="J44" s="49"/>
     </row>
-    <row r="45" spans="1:13" ht="17" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:13" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C45" s="27"/>
       <c r="D45" s="28"/>
       <c r="E45" s="50" t="s">
@@ -3255,7 +3317,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:13" ht="17" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:13" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="E46" s="50" t="s">
         <v>22</v>
       </c>
@@ -3272,7 +3334,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:13" x14ac:dyDescent="0.2">
       <c r="E47" s="50" t="s">
         <v>26</v>
       </c>
@@ -3283,7 +3345,7 @@
       <c r="H47" s="47"/>
       <c r="I47" s="47"/>
     </row>
-    <row r="48" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:13" x14ac:dyDescent="0.2">
       <c r="C48" s="57" t="s">
         <v>35</v>
       </c>
@@ -3297,7 +3359,7 @@
       <c r="H48" s="47"/>
       <c r="I48" s="47"/>
     </row>
-    <row r="49" spans="3:9" x14ac:dyDescent="0.3">
+    <row r="49" spans="3:9" x14ac:dyDescent="0.2">
       <c r="C49" s="27" t="s">
         <v>36</v>
       </c>
@@ -3311,199 +3373,199 @@
       <c r="H49" s="47"/>
       <c r="I49" s="47"/>
     </row>
-    <row r="50" spans="3:9" x14ac:dyDescent="0.3">
+    <row r="50" spans="3:9" x14ac:dyDescent="0.2">
       <c r="F50" s="47"/>
       <c r="G50" s="47"/>
       <c r="H50" s="47"/>
       <c r="I50" s="47"/>
     </row>
-    <row r="51" spans="3:9" x14ac:dyDescent="0.3">
+    <row r="51" spans="3:9" x14ac:dyDescent="0.2">
       <c r="F51" s="47"/>
       <c r="G51" s="47"/>
       <c r="H51" s="47"/>
       <c r="I51" s="47"/>
     </row>
-    <row r="52" spans="3:9" x14ac:dyDescent="0.3">
+    <row r="52" spans="3:9" x14ac:dyDescent="0.2">
       <c r="F52" s="47"/>
       <c r="G52" s="47"/>
       <c r="H52" s="47"/>
       <c r="I52" s="47"/>
     </row>
-    <row r="53" spans="3:9" x14ac:dyDescent="0.3">
+    <row r="53" spans="3:9" x14ac:dyDescent="0.2">
       <c r="F53" s="47"/>
       <c r="G53" s="47"/>
       <c r="H53" s="47"/>
       <c r="I53" s="47"/>
     </row>
-    <row r="54" spans="3:9" x14ac:dyDescent="0.3">
+    <row r="54" spans="3:9" x14ac:dyDescent="0.2">
       <c r="F54" s="47"/>
       <c r="G54" s="47"/>
       <c r="H54" s="47"/>
       <c r="I54" s="47"/>
     </row>
-    <row r="55" spans="3:9" x14ac:dyDescent="0.3">
+    <row r="55" spans="3:9" x14ac:dyDescent="0.2">
       <c r="F55" s="47"/>
       <c r="G55" s="47"/>
       <c r="H55" s="47"/>
       <c r="I55" s="47"/>
     </row>
-    <row r="56" spans="3:9" x14ac:dyDescent="0.3">
+    <row r="56" spans="3:9" x14ac:dyDescent="0.2">
       <c r="F56" s="47"/>
       <c r="G56" s="47"/>
       <c r="H56" s="47"/>
       <c r="I56" s="47"/>
     </row>
-    <row r="57" spans="3:9" x14ac:dyDescent="0.3">
+    <row r="57" spans="3:9" x14ac:dyDescent="0.2">
       <c r="F57" s="47"/>
       <c r="G57" s="47"/>
       <c r="H57" s="47"/>
       <c r="I57" s="47"/>
     </row>
-    <row r="58" spans="3:9" x14ac:dyDescent="0.3">
+    <row r="58" spans="3:9" x14ac:dyDescent="0.2">
       <c r="F58" s="47"/>
       <c r="G58" s="47"/>
       <c r="H58" s="47"/>
       <c r="I58" s="47"/>
     </row>
-    <row r="59" spans="3:9" x14ac:dyDescent="0.3">
+    <row r="59" spans="3:9" x14ac:dyDescent="0.2">
       <c r="F59" s="47"/>
       <c r="G59" s="47"/>
       <c r="H59" s="47"/>
       <c r="I59" s="47"/>
     </row>
-    <row r="60" spans="3:9" x14ac:dyDescent="0.3">
+    <row r="60" spans="3:9" x14ac:dyDescent="0.2">
       <c r="F60" s="47"/>
       <c r="G60" s="47"/>
       <c r="H60" s="47"/>
       <c r="I60" s="47"/>
     </row>
-    <row r="61" spans="3:9" x14ac:dyDescent="0.3">
+    <row r="61" spans="3:9" x14ac:dyDescent="0.2">
       <c r="F61" s="47"/>
       <c r="G61" s="47"/>
       <c r="H61" s="47"/>
       <c r="I61" s="47"/>
     </row>
-    <row r="62" spans="3:9" x14ac:dyDescent="0.3">
+    <row r="62" spans="3:9" x14ac:dyDescent="0.2">
       <c r="F62" s="47"/>
       <c r="G62" s="47"/>
       <c r="H62" s="47"/>
       <c r="I62" s="47"/>
     </row>
-    <row r="63" spans="3:9" x14ac:dyDescent="0.3">
+    <row r="63" spans="3:9" x14ac:dyDescent="0.2">
       <c r="F63" s="47"/>
       <c r="G63" s="47"/>
       <c r="H63" s="47"/>
       <c r="I63" s="47"/>
     </row>
-    <row r="64" spans="3:9" x14ac:dyDescent="0.3">
+    <row r="64" spans="3:9" x14ac:dyDescent="0.2">
       <c r="F64" s="47"/>
       <c r="G64" s="47"/>
       <c r="H64" s="47"/>
       <c r="I64" s="47"/>
     </row>
-    <row r="65" spans="6:9" x14ac:dyDescent="0.3">
+    <row r="65" spans="6:9" x14ac:dyDescent="0.2">
       <c r="F65" s="47"/>
       <c r="G65" s="47"/>
       <c r="H65" s="47"/>
       <c r="I65" s="47"/>
     </row>
-    <row r="66" spans="6:9" x14ac:dyDescent="0.3">
+    <row r="66" spans="6:9" x14ac:dyDescent="0.2">
       <c r="F66" s="47"/>
       <c r="G66" s="47"/>
       <c r="H66" s="47"/>
       <c r="I66" s="47"/>
     </row>
-    <row r="67" spans="6:9" x14ac:dyDescent="0.3">
+    <row r="67" spans="6:9" x14ac:dyDescent="0.2">
       <c r="F67" s="47"/>
       <c r="G67" s="47"/>
       <c r="H67" s="47"/>
       <c r="I67" s="47"/>
     </row>
-    <row r="68" spans="6:9" x14ac:dyDescent="0.3">
+    <row r="68" spans="6:9" x14ac:dyDescent="0.2">
       <c r="F68" s="47"/>
       <c r="G68" s="47"/>
       <c r="H68" s="47"/>
       <c r="I68" s="47"/>
     </row>
-    <row r="69" spans="6:9" x14ac:dyDescent="0.3">
+    <row r="69" spans="6:9" x14ac:dyDescent="0.2">
       <c r="F69" s="47"/>
       <c r="G69" s="47"/>
       <c r="H69" s="47"/>
       <c r="I69" s="47"/>
     </row>
-    <row r="70" spans="6:9" x14ac:dyDescent="0.3">
+    <row r="70" spans="6:9" x14ac:dyDescent="0.2">
       <c r="F70" s="47"/>
       <c r="G70" s="47"/>
       <c r="H70" s="47"/>
       <c r="I70" s="47"/>
     </row>
-    <row r="71" spans="6:9" x14ac:dyDescent="0.3">
+    <row r="71" spans="6:9" x14ac:dyDescent="0.2">
       <c r="F71" s="47"/>
       <c r="G71" s="47"/>
       <c r="H71" s="47"/>
       <c r="I71" s="47"/>
     </row>
-    <row r="72" spans="6:9" x14ac:dyDescent="0.3">
+    <row r="72" spans="6:9" x14ac:dyDescent="0.2">
       <c r="F72" s="47"/>
       <c r="G72" s="47"/>
       <c r="H72" s="47"/>
       <c r="I72" s="47"/>
     </row>
-    <row r="73" spans="6:9" x14ac:dyDescent="0.3">
+    <row r="73" spans="6:9" x14ac:dyDescent="0.2">
       <c r="F73" s="47"/>
       <c r="G73" s="47"/>
       <c r="H73" s="47"/>
       <c r="I73" s="47"/>
     </row>
-    <row r="74" spans="6:9" x14ac:dyDescent="0.3">
+    <row r="74" spans="6:9" x14ac:dyDescent="0.2">
       <c r="F74" s="47"/>
       <c r="G74" s="47"/>
       <c r="H74" s="47"/>
       <c r="I74" s="47"/>
     </row>
-    <row r="75" spans="6:9" x14ac:dyDescent="0.3">
+    <row r="75" spans="6:9" x14ac:dyDescent="0.2">
       <c r="F75" s="47"/>
       <c r="G75" s="47"/>
       <c r="H75" s="47"/>
       <c r="I75" s="47"/>
     </row>
-    <row r="76" spans="6:9" x14ac:dyDescent="0.3">
+    <row r="76" spans="6:9" x14ac:dyDescent="0.2">
       <c r="F76" s="47"/>
       <c r="G76" s="47"/>
       <c r="H76" s="47"/>
       <c r="I76" s="47"/>
     </row>
-    <row r="77" spans="6:9" x14ac:dyDescent="0.3">
+    <row r="77" spans="6:9" x14ac:dyDescent="0.2">
       <c r="F77" s="47"/>
       <c r="G77" s="47"/>
       <c r="H77" s="47"/>
       <c r="I77" s="47"/>
     </row>
-    <row r="78" spans="6:9" x14ac:dyDescent="0.3">
+    <row r="78" spans="6:9" x14ac:dyDescent="0.2">
       <c r="F78" s="47"/>
       <c r="G78" s="47"/>
       <c r="H78" s="47"/>
       <c r="I78" s="47"/>
     </row>
-    <row r="79" spans="6:9" x14ac:dyDescent="0.3">
+    <row r="79" spans="6:9" x14ac:dyDescent="0.2">
       <c r="F79" s="47"/>
       <c r="G79" s="47"/>
       <c r="H79" s="47"/>
       <c r="I79" s="47"/>
     </row>
-    <row r="80" spans="6:9" x14ac:dyDescent="0.3">
+    <row r="80" spans="6:9" x14ac:dyDescent="0.2">
       <c r="F80" s="47"/>
       <c r="G80" s="47"/>
       <c r="H80" s="47"/>
       <c r="I80" s="47"/>
     </row>
-    <row r="81" spans="6:9" x14ac:dyDescent="0.3">
+    <row r="81" spans="6:9" x14ac:dyDescent="0.2">
       <c r="F81" s="47"/>
       <c r="G81" s="47"/>
       <c r="H81" s="47"/>
       <c r="I81" s="47"/>
     </row>
-    <row r="82" spans="6:9" x14ac:dyDescent="0.3">
+    <row r="82" spans="6:9" x14ac:dyDescent="0.2">
       <c r="F82" s="47"/>
       <c r="G82" s="47"/>
       <c r="H82" s="47"/>

</xml_diff>

<commit_message>
feat: cockpit with operations log, IPO auto-fill, earnings tracking
</commit_message>
<xml_diff>
--- a/docs/fakedata-reference.xlsx
+++ b/docs/fakedata-reference.xlsx
@@ -12,15 +12,16 @@
     <workbookView xWindow="0" yWindow="0" windowWidth="25605" windowHeight="10275"/>
   </bookViews>
   <sheets>
-    <sheet name="六月 (2)" sheetId="2" r:id="rId1"/>
-    <sheet name="六月" sheetId="1" r:id="rId2"/>
+    <sheet name="收益填报" sheetId="3" r:id="rId1"/>
+    <sheet name="六月 (2)" sheetId="2" r:id="rId2"/>
+    <sheet name="六月" sheetId="1" r:id="rId3"/>
   </sheets>
   <calcPr calcId="162913"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="86">
   <si>
     <t>参加活动</t>
   </si>
@@ -190,18 +191,193 @@
   <si>
     <t>5月</t>
     <phoneticPr fontId="12" type="noConversion"/>
+  </si>
+  <si>
+    <t>序号</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>开始日期</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>结束日期</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>银行/券商</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>理财产品</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>本金（万）</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>年化收益率</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>贴息</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>天数</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>收益（元）</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>备注</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>康美特与月末冲量冲突不申购</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>年化</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="等线"/>
+        <family val="3"/>
+        <charset val="134"/>
+      </rPr>
+      <t>.20</t>
+    </r>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>1.30</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>0</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="等线"/>
+        <family val="3"/>
+        <charset val="134"/>
+      </rPr>
+      <t>.55</t>
+    </r>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>申万宏源</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>杭州银行</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>江苏银行</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>未上市</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>未上市</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>金戈新材申购</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>永达股份申购</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>新瑞电子上市</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>通知存款</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>彩客科技上市</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>通知存款</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>金戈新材上市</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>国债逆回购</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>永达股份上市</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>科莱瑞迪申购</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>吉和昌申购</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>永励精密申购</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>通知存款</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>科莱瑞迪上市</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>益坤电气上市</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>益坤电气申购</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>合计</t>
+    <phoneticPr fontId="18" type="noConversion"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="176" formatCode="#,##0_ "/>
     <numFmt numFmtId="177" formatCode="0_ "/>
     <numFmt numFmtId="178" formatCode="0.00_ "/>
+    <numFmt numFmtId="182" formatCode="#,##0.00_);[Red]\(#,##0.00\)"/>
   </numFmts>
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="21">
     <font>
       <sz val="11"/>
       <name val="等线"/>
@@ -323,8 +499,28 @@
       <family val="3"/>
       <charset val="134"/>
     </font>
+    <font>
+      <sz val="9"/>
+      <name val="等线"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="等线"/>
+      <family val="3"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="等线"/>
+      <family val="3"/>
+      <charset val="134"/>
+    </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -364,6 +560,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFDEEFF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -410,7 +612,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="65">
+  <cellXfs count="77">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -605,6 +807,42 @@
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="182" fontId="14" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="182" fontId="19" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="20" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -881,8 +1119,682 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:K118"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <cols>
+    <col min="1" max="4" width="11.875" customWidth="1"/>
+    <col min="5" max="5" width="16" customWidth="1"/>
+    <col min="6" max="10" width="11.875" customWidth="1"/>
+    <col min="11" max="11" width="27.625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11">
+      <c r="A1" s="67" t="s">
+        <v>48</v>
+      </c>
+      <c r="B1" s="67" t="s">
+        <v>49</v>
+      </c>
+      <c r="C1" s="67" t="s">
+        <v>50</v>
+      </c>
+      <c r="D1" s="67" t="s">
+        <v>51</v>
+      </c>
+      <c r="E1" s="67" t="s">
+        <v>52</v>
+      </c>
+      <c r="F1" s="67" t="s">
+        <v>53</v>
+      </c>
+      <c r="G1" s="67" t="s">
+        <v>54</v>
+      </c>
+      <c r="H1" s="67" t="s">
+        <v>55</v>
+      </c>
+      <c r="I1" s="67" t="s">
+        <v>56</v>
+      </c>
+      <c r="J1" s="67" t="s">
+        <v>57</v>
+      </c>
+      <c r="K1" s="67" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11">
+      <c r="A2" s="68">
+        <v>1</v>
+      </c>
+      <c r="B2" s="69">
+        <v>46174</v>
+      </c>
+      <c r="C2" s="69">
+        <v>46176</v>
+      </c>
+      <c r="D2" s="70" t="s">
+        <v>64</v>
+      </c>
+      <c r="E2" s="70" t="s">
+        <v>69</v>
+      </c>
+      <c r="F2" s="71">
+        <v>324.25</v>
+      </c>
+      <c r="G2" s="71"/>
+      <c r="H2" s="68"/>
+      <c r="I2" s="68">
+        <v>2</v>
+      </c>
+      <c r="J2" s="71">
+        <v>0</v>
+      </c>
+      <c r="K2" s="68"/>
+    </row>
+    <row r="3" spans="1:11">
+      <c r="A3" s="68">
+        <v>2</v>
+      </c>
+      <c r="B3" s="69">
+        <v>46176</v>
+      </c>
+      <c r="C3" s="69">
+        <v>46178</v>
+      </c>
+      <c r="D3" s="70" t="s">
+        <v>64</v>
+      </c>
+      <c r="E3" s="70" t="s">
+        <v>70</v>
+      </c>
+      <c r="F3" s="71">
+        <v>324.25</v>
+      </c>
+      <c r="G3" s="71"/>
+      <c r="H3" s="68"/>
+      <c r="I3" s="68">
+        <v>2</v>
+      </c>
+      <c r="J3" s="71">
+        <v>0</v>
+      </c>
+      <c r="K3" s="68"/>
+    </row>
+    <row r="4" spans="1:11">
+      <c r="A4" s="68">
+        <v>3</v>
+      </c>
+      <c r="B4" s="69">
+        <v>46178</v>
+      </c>
+      <c r="C4" s="69">
+        <v>46178</v>
+      </c>
+      <c r="D4" s="70" t="s">
+        <v>64</v>
+      </c>
+      <c r="E4" s="70" t="s">
+        <v>71</v>
+      </c>
+      <c r="F4" s="71">
+        <v>320.85000000000002</v>
+      </c>
+      <c r="G4" s="71"/>
+      <c r="H4" s="68">
+        <v>32</v>
+      </c>
+      <c r="I4" s="68">
+        <v>0</v>
+      </c>
+      <c r="J4" s="71">
+        <v>10267.200000000001</v>
+      </c>
+      <c r="K4" s="68"/>
+    </row>
+    <row r="5" spans="1:11">
+      <c r="A5" s="68">
+        <v>4</v>
+      </c>
+      <c r="B5" s="69">
+        <v>46178</v>
+      </c>
+      <c r="C5" s="69">
+        <v>46181</v>
+      </c>
+      <c r="D5" s="70" t="s">
+        <v>65</v>
+      </c>
+      <c r="E5" s="70" t="s">
+        <v>72</v>
+      </c>
+      <c r="F5" s="71">
+        <v>324.25</v>
+      </c>
+      <c r="G5" s="71" t="s">
+        <v>61</v>
+      </c>
+      <c r="H5" s="68"/>
+      <c r="I5" s="68">
+        <v>3</v>
+      </c>
+      <c r="J5" s="71">
+        <v>324.25</v>
+      </c>
+      <c r="K5" s="68"/>
+    </row>
+    <row r="6" spans="1:11">
+      <c r="A6" s="68">
+        <v>5</v>
+      </c>
+      <c r="B6" s="69">
+        <v>46181</v>
+      </c>
+      <c r="C6" s="69">
+        <v>46181</v>
+      </c>
+      <c r="D6" s="70" t="s">
+        <v>64</v>
+      </c>
+      <c r="E6" s="70" t="s">
+        <v>73</v>
+      </c>
+      <c r="F6" s="71">
+        <v>320.85000000000002</v>
+      </c>
+      <c r="G6" s="71"/>
+      <c r="H6" s="68">
+        <v>8</v>
+      </c>
+      <c r="I6" s="68">
+        <v>0</v>
+      </c>
+      <c r="J6" s="71">
+        <v>2566.8000000000002</v>
+      </c>
+      <c r="K6" s="68"/>
+    </row>
+    <row r="7" spans="1:11">
+      <c r="A7" s="68">
+        <v>6</v>
+      </c>
+      <c r="B7" s="69">
+        <v>46181</v>
+      </c>
+      <c r="C7" s="69">
+        <v>46184</v>
+      </c>
+      <c r="D7" s="70" t="s">
+        <v>65</v>
+      </c>
+      <c r="E7" s="70" t="s">
+        <v>74</v>
+      </c>
+      <c r="F7" s="71">
+        <v>324.25</v>
+      </c>
+      <c r="G7" s="71" t="s">
+        <v>61</v>
+      </c>
+      <c r="H7" s="68"/>
+      <c r="I7" s="68">
+        <v>3</v>
+      </c>
+      <c r="J7" s="71">
+        <v>324.25</v>
+      </c>
+      <c r="K7" s="68"/>
+    </row>
+    <row r="8" spans="1:11">
+      <c r="A8" s="68">
+        <v>7</v>
+      </c>
+      <c r="B8" s="69">
+        <v>46184</v>
+      </c>
+      <c r="C8" s="69">
+        <v>46184</v>
+      </c>
+      <c r="D8" s="70" t="s">
+        <v>64</v>
+      </c>
+      <c r="E8" s="70" t="s">
+        <v>75</v>
+      </c>
+      <c r="F8" s="71">
+        <v>324.25</v>
+      </c>
+      <c r="G8" s="71"/>
+      <c r="H8" s="68">
+        <v>11</v>
+      </c>
+      <c r="I8" s="68">
+        <v>0</v>
+      </c>
+      <c r="J8" s="71">
+        <v>3566.75</v>
+      </c>
+      <c r="K8" s="68"/>
+    </row>
+    <row r="9" spans="1:11">
+      <c r="A9" s="68">
+        <v>8</v>
+      </c>
+      <c r="B9" s="69">
+        <v>46184</v>
+      </c>
+      <c r="C9" s="69">
+        <v>46188</v>
+      </c>
+      <c r="D9" s="70" t="s">
+        <v>64</v>
+      </c>
+      <c r="E9" s="70" t="s">
+        <v>76</v>
+      </c>
+      <c r="F9" s="71">
+        <v>324.25</v>
+      </c>
+      <c r="G9" s="71" t="s">
+        <v>62</v>
+      </c>
+      <c r="H9" s="68"/>
+      <c r="I9" s="68">
+        <v>4</v>
+      </c>
+      <c r="J9" s="71">
+        <v>468.36</v>
+      </c>
+      <c r="K9" s="68"/>
+    </row>
+    <row r="10" spans="1:11">
+      <c r="A10" s="68">
+        <v>9</v>
+      </c>
+      <c r="B10" s="69">
+        <v>46188</v>
+      </c>
+      <c r="C10" s="69">
+        <v>46188</v>
+      </c>
+      <c r="D10" s="70" t="s">
+        <v>64</v>
+      </c>
+      <c r="E10" s="70" t="s">
+        <v>77</v>
+      </c>
+      <c r="F10" s="71">
+        <v>324.25</v>
+      </c>
+      <c r="G10" s="71"/>
+      <c r="H10" s="68">
+        <v>6</v>
+      </c>
+      <c r="I10" s="68">
+        <v>0</v>
+      </c>
+      <c r="J10" s="71">
+        <v>1945.5</v>
+      </c>
+      <c r="K10" s="68"/>
+    </row>
+    <row r="11" spans="1:11">
+      <c r="A11" s="68">
+        <v>10</v>
+      </c>
+      <c r="B11" s="69">
+        <v>46188</v>
+      </c>
+      <c r="C11" s="69">
+        <v>46190</v>
+      </c>
+      <c r="D11" s="70" t="s">
+        <v>64</v>
+      </c>
+      <c r="E11" s="70" t="s">
+        <v>78</v>
+      </c>
+      <c r="F11" s="71">
+        <v>324.25</v>
+      </c>
+      <c r="G11" s="71"/>
+      <c r="H11" s="68"/>
+      <c r="I11" s="68">
+        <v>2</v>
+      </c>
+      <c r="J11" s="71">
+        <v>0</v>
+      </c>
+      <c r="K11" s="68"/>
+    </row>
+    <row r="12" spans="1:11">
+      <c r="A12" s="68">
+        <v>11</v>
+      </c>
+      <c r="B12" s="69">
+        <v>46190</v>
+      </c>
+      <c r="C12" s="69">
+        <v>46195</v>
+      </c>
+      <c r="D12" s="70" t="s">
+        <v>64</v>
+      </c>
+      <c r="E12" s="70" t="s">
+        <v>79</v>
+      </c>
+      <c r="F12" s="71">
+        <v>324.25</v>
+      </c>
+      <c r="G12" s="71"/>
+      <c r="H12" s="68"/>
+      <c r="I12" s="68">
+        <v>5</v>
+      </c>
+      <c r="J12" s="71">
+        <v>0</v>
+      </c>
+      <c r="K12" s="70" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11">
+      <c r="A13" s="68">
+        <v>12</v>
+      </c>
+      <c r="B13" s="69">
+        <v>46195</v>
+      </c>
+      <c r="C13" s="69">
+        <v>46197</v>
+      </c>
+      <c r="D13" s="70" t="s">
+        <v>64</v>
+      </c>
+      <c r="E13" s="70" t="s">
+        <v>84</v>
+      </c>
+      <c r="F13" s="71">
+        <v>324.25</v>
+      </c>
+      <c r="G13" s="71"/>
+      <c r="H13" s="68"/>
+      <c r="I13" s="68">
+        <v>2</v>
+      </c>
+      <c r="J13" s="71">
+        <v>0</v>
+      </c>
+      <c r="K13" s="68"/>
+    </row>
+    <row r="14" spans="1:11">
+      <c r="A14" s="68">
+        <v>13</v>
+      </c>
+      <c r="B14" s="69">
+        <v>46197</v>
+      </c>
+      <c r="C14" s="69">
+        <v>46199</v>
+      </c>
+      <c r="D14" s="70" t="s">
+        <v>64</v>
+      </c>
+      <c r="E14" s="70" t="s">
+        <v>80</v>
+      </c>
+      <c r="F14" s="71">
+        <v>324.25</v>
+      </c>
+      <c r="G14" s="71"/>
+      <c r="H14" s="68"/>
+      <c r="I14" s="68">
+        <v>2</v>
+      </c>
+      <c r="J14" s="71">
+        <v>0</v>
+      </c>
+      <c r="K14" s="70" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11">
+      <c r="A15" s="68">
+        <v>14</v>
+      </c>
+      <c r="B15" s="69">
+        <v>46199</v>
+      </c>
+      <c r="C15" s="69">
+        <v>46203</v>
+      </c>
+      <c r="D15" s="70" t="s">
+        <v>65</v>
+      </c>
+      <c r="E15" s="70" t="s">
+        <v>81</v>
+      </c>
+      <c r="F15" s="71">
+        <v>324.25</v>
+      </c>
+      <c r="G15" s="71" t="s">
+        <v>63</v>
+      </c>
+      <c r="H15" s="68"/>
+      <c r="I15" s="68">
+        <v>4</v>
+      </c>
+      <c r="J15" s="71">
+        <v>198.15</v>
+      </c>
+      <c r="K15" s="68"/>
+    </row>
+    <row r="16" spans="1:11">
+      <c r="A16" s="68">
+        <v>15</v>
+      </c>
+      <c r="B16" s="69">
+        <v>46202</v>
+      </c>
+      <c r="C16" s="69">
+        <v>46202</v>
+      </c>
+      <c r="D16" s="70" t="s">
+        <v>64</v>
+      </c>
+      <c r="E16" s="70" t="s">
+        <v>82</v>
+      </c>
+      <c r="F16" s="71">
+        <v>324.25</v>
+      </c>
+      <c r="G16" s="71"/>
+      <c r="H16" s="68">
+        <v>22</v>
+      </c>
+      <c r="I16" s="68">
+        <v>0</v>
+      </c>
+      <c r="J16" s="71">
+        <v>7133.5</v>
+      </c>
+      <c r="K16" s="68"/>
+    </row>
+    <row r="17" spans="1:11">
+      <c r="A17" s="68">
+        <v>16</v>
+      </c>
+      <c r="B17" s="69">
+        <v>46203</v>
+      </c>
+      <c r="C17" s="69">
+        <v>46203</v>
+      </c>
+      <c r="D17" s="70" t="s">
+        <v>64</v>
+      </c>
+      <c r="E17" s="70" t="s">
+        <v>83</v>
+      </c>
+      <c r="F17" s="71">
+        <v>324.25</v>
+      </c>
+      <c r="G17" s="71"/>
+      <c r="H17" s="68">
+        <v>6</v>
+      </c>
+      <c r="I17" s="68">
+        <v>0</v>
+      </c>
+      <c r="J17" s="71">
+        <v>1945.5</v>
+      </c>
+      <c r="K17" s="68"/>
+    </row>
+    <row r="18" spans="1:11">
+      <c r="A18" s="68">
+        <v>17</v>
+      </c>
+      <c r="B18" s="69">
+        <v>46203</v>
+      </c>
+      <c r="C18" s="69">
+        <v>46204</v>
+      </c>
+      <c r="D18" s="70" t="s">
+        <v>66</v>
+      </c>
+      <c r="E18" s="70" t="s">
+        <v>74</v>
+      </c>
+      <c r="F18" s="71">
+        <v>324.25</v>
+      </c>
+      <c r="G18" s="71" t="s">
+        <v>63</v>
+      </c>
+      <c r="H18" s="68">
+        <v>15</v>
+      </c>
+      <c r="I18" s="68">
+        <v>1</v>
+      </c>
+      <c r="J18" s="71">
+        <v>4913.29</v>
+      </c>
+      <c r="K18" s="70" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11">
+      <c r="A19" s="72"/>
+      <c r="B19" s="72"/>
+      <c r="C19" s="72"/>
+      <c r="D19" s="72"/>
+      <c r="E19" s="72"/>
+      <c r="F19" s="72"/>
+      <c r="G19" s="73" t="s">
+        <v>85</v>
+      </c>
+      <c r="H19" s="73">
+        <f>SUM(H2:H18)</f>
+        <v>100</v>
+      </c>
+      <c r="I19" s="73">
+        <f>SUM(I2:I18)</f>
+        <v>30</v>
+      </c>
+      <c r="J19" s="74">
+        <f>SUM(J2:J18)</f>
+        <v>33653.550000000003</v>
+      </c>
+      <c r="K19" s="72"/>
+    </row>
+    <row r="20" spans="1:11">
+      <c r="A20" s="68"/>
+      <c r="B20" s="68"/>
+      <c r="C20" s="68"/>
+      <c r="D20" s="68"/>
+      <c r="E20" s="68"/>
+      <c r="F20" s="68"/>
+      <c r="G20" s="68"/>
+      <c r="H20" s="68"/>
+      <c r="I20" s="75" t="s">
+        <v>60</v>
+      </c>
+      <c r="J20" s="76">
+        <v>0.1245</v>
+      </c>
+      <c r="K20" s="68"/>
+    </row>
+    <row r="24" spans="1:11">
+      <c r="A24" s="65"/>
+    </row>
+    <row r="30" spans="1:11">
+      <c r="A30" s="65"/>
+    </row>
+    <row r="31" spans="1:11">
+      <c r="A31" s="65"/>
+    </row>
+    <row r="43" spans="1:1">
+      <c r="A43" s="65"/>
+    </row>
+    <row r="48" spans="1:1">
+      <c r="A48" s="65"/>
+    </row>
+    <row r="51" spans="1:1">
+      <c r="A51" s="65"/>
+    </row>
+    <row r="52" spans="1:1">
+      <c r="A52" s="65"/>
+    </row>
+    <row r="59" spans="1:1">
+      <c r="A59" s="65"/>
+    </row>
+    <row r="60" spans="1:1">
+      <c r="A60" s="65"/>
+    </row>
+    <row r="70" spans="1:1">
+      <c r="A70" s="65"/>
+    </row>
+    <row r="75" spans="1:1">
+      <c r="A75" s="65"/>
+    </row>
+    <row r="80" spans="1:1">
+      <c r="A80" s="65"/>
+    </row>
+    <row r="85" spans="1:1">
+      <c r="A85" s="65"/>
+    </row>
+    <row r="88" spans="1:1">
+      <c r="A88" s="65"/>
+    </row>
+    <row r="104" spans="1:1">
+      <c r="A104" s="65"/>
+    </row>
+    <row r="105" spans="1:1">
+      <c r="A105" s="65"/>
+    </row>
+    <row r="112" spans="1:1">
+      <c r="A112" s="65"/>
+    </row>
+    <row r="113" spans="1:1">
+      <c r="A113" s="65"/>
+    </row>
+    <row r="118" spans="1:1">
+      <c r="A118" s="66"/>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="18" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A3:O80"/>
-  <sheetFormatPr defaultColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="10" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="12.125" customWidth="1"/>
     <col min="2" max="2" width="5.125" style="11" customWidth="1"/>
@@ -900,7 +1812,7 @@
     <col min="15" max="15" width="10.625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:15" s="1" customFormat="1" ht="107.45" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:15" s="1" customFormat="1" ht="107.45" customHeight="1">
       <c r="B3" s="9"/>
       <c r="C3" s="10" t="s">
         <v>0</v>
@@ -921,7 +1833,7 @@
       <c r="M3" s="30"/>
       <c r="N3" s="30"/>
     </row>
-    <row r="4" spans="1:15" s="2" customFormat="1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:15" s="2" customFormat="1" ht="17.100000000000001" customHeight="1">
       <c r="B4" s="11"/>
       <c r="C4" s="12" t="s">
         <v>31</v>
@@ -952,7 +1864,7 @@
       </c>
       <c r="N4" s="32"/>
     </row>
-    <row r="5" spans="1:15" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:15" ht="17.100000000000001" customHeight="1">
       <c r="C5" s="13" t="s">
         <v>32</v>
       </c>
@@ -972,7 +1884,7 @@
       <c r="J5" s="33"/>
       <c r="K5" s="33"/>
     </row>
-    <row r="6" spans="1:15" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:15" ht="17.100000000000001" customHeight="1">
       <c r="B6" s="15"/>
       <c r="C6" s="16" t="s">
         <v>4</v>
@@ -990,7 +1902,7 @@
       <c r="J6" s="34"/>
       <c r="K6" s="34"/>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:15">
       <c r="B7" s="64" t="s">
         <v>28</v>
       </c>
@@ -1018,7 +1930,7 @@
         <v>7001241</v>
       </c>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:15">
       <c r="B8" s="64" t="s">
         <v>29</v>
       </c>
@@ -1044,7 +1956,7 @@
         <v>16710312</v>
       </c>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:15">
       <c r="B9" s="64" t="s">
         <v>8</v>
       </c>
@@ -1070,7 +1982,7 @@
         <v>18010379</v>
       </c>
     </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:15">
       <c r="B10" s="64" t="s">
         <v>9</v>
       </c>
@@ -1100,7 +2012,7 @@
       </c>
       <c r="O10" s="51"/>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:15">
       <c r="B11" s="64" t="s">
         <v>10</v>
       </c>
@@ -1126,7 +2038,7 @@
         <v>27650363</v>
       </c>
     </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:15">
       <c r="B12" s="64" t="s">
         <v>11</v>
       </c>
@@ -1154,7 +2066,7 @@
       <c r="M12" s="59"/>
       <c r="O12" s="35"/>
     </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:15">
       <c r="B13" s="64" t="s">
         <v>5</v>
       </c>
@@ -1181,7 +2093,7 @@
       </c>
       <c r="N13" s="62"/>
     </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:15">
       <c r="B14" s="64" t="s">
         <v>6</v>
       </c>
@@ -1207,7 +2119,7 @@
         <v>10750529</v>
       </c>
     </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:15">
       <c r="A15" s="57" t="s">
         <v>25</v>
       </c>
@@ -1236,7 +2148,7 @@
         <v>15750529</v>
       </c>
     </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:15">
       <c r="B16" s="64" t="s">
         <v>8</v>
       </c>
@@ -1263,7 +2175,7 @@
         <v>18060433</v>
       </c>
     </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:12">
       <c r="B17" s="64" t="s">
         <v>9</v>
       </c>
@@ -1287,7 +2199,7 @@
         <v>7008404</v>
       </c>
     </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:12">
       <c r="B18" s="64" t="s">
         <v>10</v>
       </c>
@@ -1311,7 +2223,7 @@
         <v>17478230</v>
       </c>
     </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:12">
       <c r="B19" s="64" t="s">
         <v>11</v>
       </c>
@@ -1335,7 +2247,7 @@
         <v>17489277</v>
       </c>
     </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:12">
       <c r="A20" s="19"/>
       <c r="B20" s="64" t="s">
         <v>5</v>
@@ -1360,7 +2272,7 @@
         <v>17489277</v>
       </c>
     </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:12">
       <c r="A21" s="19"/>
       <c r="B21" s="64" t="s">
         <v>6</v>
@@ -1387,7 +2299,7 @@
         <v>13319277</v>
       </c>
     </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:12">
       <c r="A22" s="19"/>
       <c r="B22" s="64" t="s">
         <v>7</v>
@@ -1412,7 +2324,7 @@
         <v>11179277</v>
       </c>
     </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:12">
       <c r="A23" s="19"/>
       <c r="B23" s="64" t="s">
         <v>8</v>
@@ -1441,7 +2353,7 @@
         <v>7119277</v>
       </c>
     </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:12">
       <c r="A24" s="19"/>
       <c r="B24" s="64" t="s">
         <v>9</v>
@@ -1468,7 +2380,7 @@
         <v>17589277</v>
       </c>
     </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:12">
       <c r="A25" s="19"/>
       <c r="B25" s="64" t="s">
         <v>10</v>
@@ -1495,7 +2407,7 @@
         <v>17589277</v>
       </c>
     </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:12">
       <c r="A26" s="19"/>
       <c r="B26" s="64" t="s">
         <v>11</v>
@@ -1522,7 +2434,7 @@
         <v>17589277</v>
       </c>
     </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:12">
       <c r="A27" s="19"/>
       <c r="B27" s="64" t="s">
         <v>5</v>
@@ -1549,7 +2461,7 @@
         <v>17589277</v>
       </c>
     </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:12">
       <c r="A28" s="19"/>
       <c r="B28" s="64" t="s">
         <v>6</v>
@@ -1576,7 +2488,7 @@
         <v>7019277</v>
       </c>
     </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:12">
       <c r="A29" s="19"/>
       <c r="B29" s="64" t="s">
         <v>7</v>
@@ -1605,7 +2517,7 @@
         <v>18719277</v>
       </c>
     </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:12">
       <c r="A30" s="19"/>
       <c r="B30" s="64" t="s">
         <v>8</v>
@@ -1632,7 +2544,7 @@
         <v>7019277</v>
       </c>
     </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:12">
       <c r="B31" s="64" t="s">
         <v>9</v>
       </c>
@@ -1656,7 +2568,7 @@
         <v>20219277</v>
       </c>
     </row>
-    <row r="32" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:12">
       <c r="B32" s="64" t="s">
         <v>10</v>
       </c>
@@ -1682,7 +2594,7 @@
         <v>17609277</v>
       </c>
     </row>
-    <row r="33" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:14">
       <c r="B33" s="64" t="s">
         <v>11</v>
       </c>
@@ -1709,7 +2621,7 @@
         <v>18199277</v>
       </c>
     </row>
-    <row r="34" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:14">
       <c r="B34" s="64" t="s">
         <v>5</v>
       </c>
@@ -1735,7 +2647,7 @@
         <v>18379277</v>
       </c>
     </row>
-    <row r="35" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:14">
       <c r="B35" s="64" t="s">
         <v>6</v>
       </c>
@@ -1761,7 +2673,7 @@
         <v>7019277</v>
       </c>
     </row>
-    <row r="36" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:14">
       <c r="B36" s="64" t="s">
         <v>7</v>
       </c>
@@ -1785,7 +2697,7 @@
         <v>14789277</v>
       </c>
     </row>
-    <row r="37" spans="1:14" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:14" ht="17.100000000000001" customHeight="1">
       <c r="B37" s="15"/>
       <c r="C37" s="20" t="s">
         <v>12</v>
@@ -1814,7 +2726,7 @@
       </c>
       <c r="K37" s="38"/>
     </row>
-    <row r="38" spans="1:14" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:14" ht="17.100000000000001" customHeight="1">
       <c r="B38" s="15"/>
       <c r="C38" s="21" t="s">
         <v>13</v>
@@ -1843,7 +2755,7 @@
       </c>
       <c r="K38" s="40"/>
     </row>
-    <row r="39" spans="1:14" s="3" customFormat="1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:14" s="3" customFormat="1" ht="17.100000000000001" customHeight="1">
       <c r="B39" s="15"/>
       <c r="C39" s="22" t="s">
         <v>14</v>
@@ -1878,7 +2790,7 @@
       </c>
       <c r="N39" s="52"/>
     </row>
-    <row r="40" spans="1:14" s="4" customFormat="1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:14" s="4" customFormat="1" ht="17.100000000000001" customHeight="1">
       <c r="B40" s="11"/>
       <c r="C40" s="23" t="s">
         <v>15</v>
@@ -1897,7 +2809,7 @@
       <c r="M40" s="53"/>
       <c r="N40" s="53"/>
     </row>
-    <row r="41" spans="1:14" s="5" customFormat="1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:14" s="5" customFormat="1" ht="17.100000000000001" customHeight="1">
       <c r="B41" s="11"/>
       <c r="C41" s="10" t="s">
         <v>16</v>
@@ -1917,7 +2829,7 @@
       <c r="M41" s="54"/>
       <c r="N41" s="54"/>
     </row>
-    <row r="42" spans="1:14" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:14" ht="24.95" customHeight="1">
       <c r="F42" s="47"/>
       <c r="G42" s="47"/>
       <c r="H42" s="47"/>
@@ -1929,7 +2841,7 @@
         <v>193.6</v>
       </c>
     </row>
-    <row r="43" spans="1:14" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:14" ht="17.100000000000001" customHeight="1">
       <c r="A43" s="24"/>
       <c r="B43" s="25"/>
       <c r="C43" s="8" t="s">
@@ -1957,7 +2869,7 @@
       <c r="K43" s="49"/>
       <c r="M43" s="49"/>
     </row>
-    <row r="44" spans="1:14" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:14" ht="17.100000000000001" customHeight="1">
       <c r="C44" s="27" t="s">
         <v>19</v>
       </c>
@@ -1984,7 +2896,7 @@
       </c>
       <c r="K44" s="49"/>
     </row>
-    <row r="45" spans="1:14" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:14" ht="17.100000000000001" customHeight="1">
       <c r="C45" s="27"/>
       <c r="D45" s="28"/>
       <c r="E45" s="50" t="s">
@@ -2006,7 +2918,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:14" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:14" ht="17.100000000000001" customHeight="1">
       <c r="E46" s="50" t="s">
         <v>22</v>
       </c>
@@ -2024,7 +2936,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:14">
       <c r="E47" s="50" t="s">
         <v>26</v>
       </c>
@@ -2036,7 +2948,7 @@
       <c r="I47" s="47"/>
       <c r="J47" s="47"/>
     </row>
-    <row r="48" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:14">
       <c r="C48" s="57" t="s">
         <v>35</v>
       </c>
@@ -2051,7 +2963,7 @@
       <c r="I48" s="47"/>
       <c r="J48" s="47"/>
     </row>
-    <row r="49" spans="3:14" x14ac:dyDescent="0.2">
+    <row r="49" spans="3:14">
       <c r="C49" s="27" t="s">
         <v>36</v>
       </c>
@@ -2066,84 +2978,84 @@
       <c r="I49" s="47"/>
       <c r="J49" s="47"/>
     </row>
-    <row r="50" spans="3:14" x14ac:dyDescent="0.2">
+    <row r="50" spans="3:14">
       <c r="F50" s="47"/>
       <c r="G50" s="47"/>
       <c r="H50" s="47"/>
       <c r="I50" s="47"/>
       <c r="J50" s="47"/>
     </row>
-    <row r="51" spans="3:14" x14ac:dyDescent="0.2">
+    <row r="51" spans="3:14">
       <c r="F51" s="47"/>
       <c r="G51" s="47"/>
       <c r="H51" s="47"/>
       <c r="I51" s="47"/>
       <c r="J51" s="47"/>
     </row>
-    <row r="52" spans="3:14" x14ac:dyDescent="0.2">
+    <row r="52" spans="3:14">
       <c r="F52" s="47"/>
       <c r="G52" s="47"/>
       <c r="H52" s="47"/>
       <c r="I52" s="47"/>
       <c r="J52" s="47"/>
     </row>
-    <row r="53" spans="3:14" x14ac:dyDescent="0.2">
+    <row r="53" spans="3:14">
       <c r="F53" s="47"/>
       <c r="G53" s="47"/>
       <c r="H53" s="47"/>
       <c r="I53" s="47"/>
       <c r="J53" s="47"/>
     </row>
-    <row r="54" spans="3:14" x14ac:dyDescent="0.2">
+    <row r="54" spans="3:14">
       <c r="F54" s="47"/>
       <c r="G54" s="47"/>
       <c r="H54" s="47"/>
       <c r="I54" s="47"/>
       <c r="J54" s="47"/>
     </row>
-    <row r="55" spans="3:14" x14ac:dyDescent="0.2">
+    <row r="55" spans="3:14">
       <c r="F55" s="47"/>
       <c r="G55" s="47"/>
       <c r="H55" s="47"/>
       <c r="I55" s="47"/>
       <c r="J55" s="47"/>
     </row>
-    <row r="56" spans="3:14" x14ac:dyDescent="0.2">
+    <row r="56" spans="3:14">
       <c r="F56" s="47"/>
       <c r="G56" s="47"/>
       <c r="H56" s="47"/>
       <c r="I56" s="47"/>
       <c r="J56" s="47"/>
     </row>
-    <row r="57" spans="3:14" x14ac:dyDescent="0.2">
+    <row r="57" spans="3:14">
       <c r="F57" s="47"/>
       <c r="G57" s="47"/>
       <c r="H57" s="47"/>
       <c r="I57" s="47"/>
       <c r="J57" s="47"/>
     </row>
-    <row r="58" spans="3:14" x14ac:dyDescent="0.2">
+    <row r="58" spans="3:14">
       <c r="F58" s="47"/>
       <c r="G58" s="47"/>
       <c r="H58" s="47"/>
       <c r="I58" s="47"/>
       <c r="J58" s="47"/>
     </row>
-    <row r="59" spans="3:14" x14ac:dyDescent="0.2">
+    <row r="59" spans="3:14">
       <c r="F59" s="47"/>
       <c r="G59" s="47"/>
       <c r="H59" s="47"/>
       <c r="I59" s="47"/>
       <c r="J59" s="47"/>
     </row>
-    <row r="60" spans="3:14" x14ac:dyDescent="0.2">
+    <row r="60" spans="3:14">
       <c r="F60" s="47"/>
       <c r="G60" s="47"/>
       <c r="H60" s="47"/>
       <c r="I60" s="47"/>
       <c r="J60" s="47"/>
     </row>
-    <row r="61" spans="3:14" x14ac:dyDescent="0.2">
+    <row r="61" spans="3:14">
       <c r="D61" s="47"/>
       <c r="E61" s="47"/>
       <c r="F61" s="47"/>
@@ -2155,7 +3067,7 @@
       <c r="M61"/>
       <c r="N61"/>
     </row>
-    <row r="62" spans="3:14" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="62" spans="3:14" ht="15.75">
       <c r="C62" s="12" t="s">
         <v>47</v>
       </c>
@@ -2181,7 +3093,7 @@
       <c r="M62"/>
       <c r="N62"/>
     </row>
-    <row r="63" spans="3:14" x14ac:dyDescent="0.2">
+    <row r="63" spans="3:14">
       <c r="C63" s="18">
         <v>46145</v>
       </c>
@@ -2201,7 +3113,7 @@
       <c r="M63"/>
       <c r="N63"/>
     </row>
-    <row r="64" spans="3:14" x14ac:dyDescent="0.2">
+    <row r="64" spans="3:14">
       <c r="C64" s="18">
         <v>46146</v>
       </c>
@@ -2221,7 +3133,7 @@
       <c r="M64"/>
       <c r="N64"/>
     </row>
-    <row r="65" spans="3:14" x14ac:dyDescent="0.2">
+    <row r="65" spans="3:14">
       <c r="C65" s="18">
         <v>46147</v>
       </c>
@@ -2241,7 +3153,7 @@
       <c r="M65"/>
       <c r="N65"/>
     </row>
-    <row r="66" spans="3:14" x14ac:dyDescent="0.2">
+    <row r="66" spans="3:14">
       <c r="D66" s="47"/>
       <c r="E66" s="47"/>
       <c r="F66" s="47"/>
@@ -2253,7 +3165,7 @@
       <c r="M66"/>
       <c r="N66"/>
     </row>
-    <row r="67" spans="3:14" x14ac:dyDescent="0.2">
+    <row r="67" spans="3:14">
       <c r="D67" s="47"/>
       <c r="E67" s="47"/>
       <c r="F67" s="47"/>
@@ -2265,91 +3177,91 @@
       <c r="M67"/>
       <c r="N67"/>
     </row>
-    <row r="68" spans="3:14" x14ac:dyDescent="0.2">
+    <row r="68" spans="3:14">
       <c r="F68" s="47"/>
       <c r="G68" s="47"/>
       <c r="H68" s="47"/>
       <c r="I68" s="47"/>
       <c r="J68" s="47"/>
     </row>
-    <row r="69" spans="3:14" x14ac:dyDescent="0.2">
+    <row r="69" spans="3:14">
       <c r="F69" s="47"/>
       <c r="G69" s="47"/>
       <c r="H69" s="47"/>
       <c r="I69" s="47"/>
       <c r="J69" s="47"/>
     </row>
-    <row r="70" spans="3:14" x14ac:dyDescent="0.2">
+    <row r="70" spans="3:14">
       <c r="F70" s="47"/>
       <c r="G70" s="47"/>
       <c r="H70" s="47"/>
       <c r="I70" s="47"/>
       <c r="J70" s="47"/>
     </row>
-    <row r="71" spans="3:14" x14ac:dyDescent="0.2">
+    <row r="71" spans="3:14">
       <c r="F71" s="47"/>
       <c r="G71" s="47"/>
       <c r="H71" s="47"/>
       <c r="I71" s="47"/>
       <c r="J71" s="47"/>
     </row>
-    <row r="72" spans="3:14" x14ac:dyDescent="0.2">
+    <row r="72" spans="3:14">
       <c r="F72" s="47"/>
       <c r="G72" s="47"/>
       <c r="H72" s="47"/>
       <c r="I72" s="47"/>
       <c r="J72" s="47"/>
     </row>
-    <row r="73" spans="3:14" x14ac:dyDescent="0.2">
+    <row r="73" spans="3:14">
       <c r="F73" s="47"/>
       <c r="G73" s="47"/>
       <c r="H73" s="47"/>
       <c r="I73" s="47"/>
       <c r="J73" s="47"/>
     </row>
-    <row r="74" spans="3:14" x14ac:dyDescent="0.2">
+    <row r="74" spans="3:14">
       <c r="F74" s="47"/>
       <c r="G74" s="47"/>
       <c r="H74" s="47"/>
       <c r="I74" s="47"/>
       <c r="J74" s="47"/>
     </row>
-    <row r="75" spans="3:14" x14ac:dyDescent="0.2">
+    <row r="75" spans="3:14">
       <c r="F75" s="47"/>
       <c r="G75" s="47"/>
       <c r="H75" s="47"/>
       <c r="I75" s="47"/>
       <c r="J75" s="47"/>
     </row>
-    <row r="76" spans="3:14" x14ac:dyDescent="0.2">
+    <row r="76" spans="3:14">
       <c r="F76" s="47"/>
       <c r="G76" s="47"/>
       <c r="H76" s="47"/>
       <c r="I76" s="47"/>
       <c r="J76" s="47"/>
     </row>
-    <row r="77" spans="3:14" x14ac:dyDescent="0.2">
+    <row r="77" spans="3:14">
       <c r="F77" s="47"/>
       <c r="G77" s="47"/>
       <c r="H77" s="47"/>
       <c r="I77" s="47"/>
       <c r="J77" s="47"/>
     </row>
-    <row r="78" spans="3:14" x14ac:dyDescent="0.2">
+    <row r="78" spans="3:14">
       <c r="F78" s="47"/>
       <c r="G78" s="47"/>
       <c r="H78" s="47"/>
       <c r="I78" s="47"/>
       <c r="J78" s="47"/>
     </row>
-    <row r="79" spans="3:14" x14ac:dyDescent="0.2">
+    <row r="79" spans="3:14">
       <c r="F79" s="47"/>
       <c r="G79" s="47"/>
       <c r="H79" s="47"/>
       <c r="I79" s="47"/>
       <c r="J79" s="47"/>
     </row>
-    <row r="80" spans="3:14" x14ac:dyDescent="0.2">
+    <row r="80" spans="3:14">
       <c r="F80" s="47"/>
       <c r="G80" s="47"/>
       <c r="H80" s="47"/>
@@ -2363,10 +3275,10 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A3:N82"/>
-  <sheetFormatPr defaultColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="10" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="12.125" customWidth="1"/>
     <col min="2" max="2" width="5.125" style="6" customWidth="1"/>
@@ -2384,7 +3296,7 @@
     <col min="14" max="14" width="10.625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:14" s="1" customFormat="1" ht="107.45" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:14" s="1" customFormat="1" ht="107.45" customHeight="1">
       <c r="B3" s="9"/>
       <c r="C3" s="10" t="s">
         <v>0</v>
@@ -2404,7 +3316,7 @@
       <c r="L3" s="30"/>
       <c r="M3" s="30"/>
     </row>
-    <row r="4" spans="1:14" s="2" customFormat="1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:14" s="2" customFormat="1" ht="17.100000000000001" customHeight="1">
       <c r="B4" s="11"/>
       <c r="C4" s="12" t="s">
         <v>31</v>
@@ -2430,7 +3342,7 @@
       </c>
       <c r="M4" s="32"/>
     </row>
-    <row r="5" spans="1:14" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:14" ht="17.100000000000001" customHeight="1">
       <c r="C5" s="13" t="s">
         <v>32</v>
       </c>
@@ -2446,7 +3358,7 @@
       <c r="I5" s="33"/>
       <c r="J5" s="33"/>
     </row>
-    <row r="6" spans="1:14" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:14" ht="17.100000000000001" customHeight="1">
       <c r="B6" s="15"/>
       <c r="C6" s="16" t="s">
         <v>4</v>
@@ -2463,7 +3375,7 @@
       <c r="I6" s="34"/>
       <c r="J6" s="34"/>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:14">
       <c r="B7" s="64" t="s">
         <v>28</v>
       </c>
@@ -2488,7 +3400,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:14">
       <c r="B8" s="64" t="s">
         <v>29</v>
       </c>
@@ -2511,7 +3423,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:14">
       <c r="B9" s="64" t="s">
         <v>8</v>
       </c>
@@ -2536,7 +3448,7 @@
         <v>10800000</v>
       </c>
     </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:14">
       <c r="B10" s="64" t="s">
         <v>9</v>
       </c>
@@ -2561,7 +3473,7 @@
       <c r="L10" s="59"/>
       <c r="N10" s="51"/>
     </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:14">
       <c r="B11" s="64" t="s">
         <v>10</v>
       </c>
@@ -2584,7 +3496,7 @@
         <v>10350000</v>
       </c>
     </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:14">
       <c r="B12" s="64" t="s">
         <v>11</v>
       </c>
@@ -2609,7 +3521,7 @@
       <c r="L12" s="59"/>
       <c r="N12" s="35"/>
     </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:14">
       <c r="B13" s="64" t="s">
         <v>5</v>
       </c>
@@ -2633,7 +3545,7 @@
       </c>
       <c r="M13" s="62"/>
     </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:14">
       <c r="B14" s="64" t="s">
         <v>6</v>
       </c>
@@ -2654,7 +3566,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:14">
       <c r="A15" s="57" t="s">
         <v>25</v>
       </c>
@@ -2678,7 +3590,7 @@
         <v>10350000</v>
       </c>
     </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:14">
       <c r="B16" s="64" t="s">
         <v>8</v>
       </c>
@@ -2699,7 +3611,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:11">
       <c r="B17" s="64" t="s">
         <v>9</v>
       </c>
@@ -2720,7 +3632,7 @@
         <v>10350000</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:11">
       <c r="B18" s="64" t="s">
         <v>10</v>
       </c>
@@ -2741,7 +3653,7 @@
         <v>10350000</v>
       </c>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:11">
       <c r="B19" s="64" t="s">
         <v>11</v>
       </c>
@@ -2762,7 +3674,7 @@
         <v>10350000</v>
       </c>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:11">
       <c r="A20" s="19"/>
       <c r="B20" s="64" t="s">
         <v>5</v>
@@ -2784,7 +3696,7 @@
         <v>10350000</v>
       </c>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:11">
       <c r="A21" s="19"/>
       <c r="B21" s="64" t="s">
         <v>6</v>
@@ -2806,7 +3718,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:11">
       <c r="A22" s="19"/>
       <c r="B22" s="64" t="s">
         <v>7</v>
@@ -2828,7 +3740,7 @@
         <v>10350000</v>
       </c>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:11">
       <c r="A23" s="19"/>
       <c r="B23" s="64" t="s">
         <v>8</v>
@@ -2850,7 +3762,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:11">
       <c r="A24" s="19"/>
       <c r="B24" s="64" t="s">
         <v>9</v>
@@ -2872,7 +3784,7 @@
         <v>10350000</v>
       </c>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:11">
       <c r="A25" s="19"/>
       <c r="B25" s="64" t="s">
         <v>10</v>
@@ -2894,7 +3806,7 @@
         <v>10350000</v>
       </c>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:11">
       <c r="A26" s="19"/>
       <c r="B26" s="64" t="s">
         <v>11</v>
@@ -2916,7 +3828,7 @@
         <v>10350000</v>
       </c>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:11">
       <c r="A27" s="19"/>
       <c r="B27" s="64" t="s">
         <v>5</v>
@@ -2938,7 +3850,7 @@
         <v>10350000</v>
       </c>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:11">
       <c r="A28" s="19"/>
       <c r="B28" s="64" t="s">
         <v>6</v>
@@ -2960,7 +3872,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:11">
       <c r="A29" s="19"/>
       <c r="B29" s="64" t="s">
         <v>7</v>
@@ -2982,7 +3894,7 @@
         <v>10350000</v>
       </c>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:11">
       <c r="A30" s="19"/>
       <c r="B30" s="64" t="s">
         <v>8</v>
@@ -3004,7 +3916,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:11">
       <c r="B31" s="64" t="s">
         <v>9</v>
       </c>
@@ -3025,7 +3937,7 @@
         <v>10350000</v>
       </c>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:11">
       <c r="B32" s="64" t="s">
         <v>10</v>
       </c>
@@ -3046,7 +3958,7 @@
         <v>10350000</v>
       </c>
     </row>
-    <row r="33" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:13">
       <c r="B33" s="64" t="s">
         <v>11</v>
       </c>
@@ -3067,7 +3979,7 @@
         <v>10350000</v>
       </c>
     </row>
-    <row r="34" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:13">
       <c r="B34" s="64" t="s">
         <v>5</v>
       </c>
@@ -3088,7 +4000,7 @@
         <v>10350000</v>
       </c>
     </row>
-    <row r="35" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:13">
       <c r="B35" s="64" t="s">
         <v>6</v>
       </c>
@@ -3109,7 +4021,7 @@
         <v>10350000</v>
       </c>
     </row>
-    <row r="36" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:13">
       <c r="B36" s="64" t="s">
         <v>7</v>
       </c>
@@ -3130,7 +4042,7 @@
         <v>10350000</v>
       </c>
     </row>
-    <row r="37" spans="1:13" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:13" ht="17.100000000000001" customHeight="1">
       <c r="B37" s="15"/>
       <c r="C37" s="20" t="s">
         <v>12</v>
@@ -3155,7 +4067,7 @@
       </c>
       <c r="J37" s="38"/>
     </row>
-    <row r="38" spans="1:13" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:13" ht="17.100000000000001" customHeight="1">
       <c r="B38" s="15"/>
       <c r="C38" s="21" t="s">
         <v>13</v>
@@ -3180,7 +4092,7 @@
       </c>
       <c r="J38" s="40"/>
     </row>
-    <row r="39" spans="1:13" s="3" customFormat="1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:13" s="3" customFormat="1" ht="17.100000000000001" customHeight="1">
       <c r="B39" s="15"/>
       <c r="C39" s="22" t="s">
         <v>14</v>
@@ -3208,7 +4120,7 @@
       <c r="L39" s="52"/>
       <c r="M39" s="52"/>
     </row>
-    <row r="40" spans="1:13" s="4" customFormat="1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:13" s="4" customFormat="1" ht="17.100000000000001" customHeight="1">
       <c r="B40" s="11"/>
       <c r="C40" s="23" t="s">
         <v>15</v>
@@ -3226,7 +4138,7 @@
       <c r="L40" s="53"/>
       <c r="M40" s="53"/>
     </row>
-    <row r="41" spans="1:13" s="5" customFormat="1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:13" s="5" customFormat="1" ht="17.100000000000001" customHeight="1">
       <c r="B41" s="11"/>
       <c r="C41" s="10" t="s">
         <v>16</v>
@@ -3242,7 +4154,7 @@
       <c r="L41" s="54"/>
       <c r="M41" s="54"/>
     </row>
-    <row r="42" spans="1:13" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:13" ht="24.95" customHeight="1">
       <c r="F42" s="47"/>
       <c r="G42" s="47"/>
       <c r="H42" s="47"/>
@@ -3253,7 +4165,7 @@
         <v>193.6</v>
       </c>
     </row>
-    <row r="43" spans="1:13" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:13" ht="17.100000000000001" customHeight="1">
       <c r="A43" s="24"/>
       <c r="B43" s="25"/>
       <c r="C43" s="8" t="s">
@@ -3276,7 +4188,7 @@
       <c r="J43" s="49"/>
       <c r="L43" s="49"/>
     </row>
-    <row r="44" spans="1:13" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:13" ht="17.100000000000001" customHeight="1">
       <c r="C44" s="27" t="s">
         <v>19</v>
       </c>
@@ -3299,7 +4211,7 @@
       </c>
       <c r="J44" s="49"/>
     </row>
-    <row r="45" spans="1:13" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:13" ht="17.100000000000001" customHeight="1">
       <c r="C45" s="27"/>
       <c r="D45" s="28"/>
       <c r="E45" s="50" t="s">
@@ -3317,7 +4229,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:13" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:13" ht="17.100000000000001" customHeight="1">
       <c r="E46" s="50" t="s">
         <v>22</v>
       </c>
@@ -3334,7 +4246,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:13">
       <c r="E47" s="50" t="s">
         <v>26</v>
       </c>
@@ -3345,7 +4257,7 @@
       <c r="H47" s="47"/>
       <c r="I47" s="47"/>
     </row>
-    <row r="48" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:13">
       <c r="C48" s="57" t="s">
         <v>35</v>
       </c>
@@ -3359,7 +4271,7 @@
       <c r="H48" s="47"/>
       <c r="I48" s="47"/>
     </row>
-    <row r="49" spans="3:9" x14ac:dyDescent="0.2">
+    <row r="49" spans="3:9">
       <c r="C49" s="27" t="s">
         <v>36</v>
       </c>
@@ -3373,199 +4285,199 @@
       <c r="H49" s="47"/>
       <c r="I49" s="47"/>
     </row>
-    <row r="50" spans="3:9" x14ac:dyDescent="0.2">
+    <row r="50" spans="3:9">
       <c r="F50" s="47"/>
       <c r="G50" s="47"/>
       <c r="H50" s="47"/>
       <c r="I50" s="47"/>
     </row>
-    <row r="51" spans="3:9" x14ac:dyDescent="0.2">
+    <row r="51" spans="3:9">
       <c r="F51" s="47"/>
       <c r="G51" s="47"/>
       <c r="H51" s="47"/>
       <c r="I51" s="47"/>
     </row>
-    <row r="52" spans="3:9" x14ac:dyDescent="0.2">
+    <row r="52" spans="3:9">
       <c r="F52" s="47"/>
       <c r="G52" s="47"/>
       <c r="H52" s="47"/>
       <c r="I52" s="47"/>
     </row>
-    <row r="53" spans="3:9" x14ac:dyDescent="0.2">
+    <row r="53" spans="3:9">
       <c r="F53" s="47"/>
       <c r="G53" s="47"/>
       <c r="H53" s="47"/>
       <c r="I53" s="47"/>
     </row>
-    <row r="54" spans="3:9" x14ac:dyDescent="0.2">
+    <row r="54" spans="3:9">
       <c r="F54" s="47"/>
       <c r="G54" s="47"/>
       <c r="H54" s="47"/>
       <c r="I54" s="47"/>
     </row>
-    <row r="55" spans="3:9" x14ac:dyDescent="0.2">
+    <row r="55" spans="3:9">
       <c r="F55" s="47"/>
       <c r="G55" s="47"/>
       <c r="H55" s="47"/>
       <c r="I55" s="47"/>
     </row>
-    <row r="56" spans="3:9" x14ac:dyDescent="0.2">
+    <row r="56" spans="3:9">
       <c r="F56" s="47"/>
       <c r="G56" s="47"/>
       <c r="H56" s="47"/>
       <c r="I56" s="47"/>
     </row>
-    <row r="57" spans="3:9" x14ac:dyDescent="0.2">
+    <row r="57" spans="3:9">
       <c r="F57" s="47"/>
       <c r="G57" s="47"/>
       <c r="H57" s="47"/>
       <c r="I57" s="47"/>
     </row>
-    <row r="58" spans="3:9" x14ac:dyDescent="0.2">
+    <row r="58" spans="3:9">
       <c r="F58" s="47"/>
       <c r="G58" s="47"/>
       <c r="H58" s="47"/>
       <c r="I58" s="47"/>
     </row>
-    <row r="59" spans="3:9" x14ac:dyDescent="0.2">
+    <row r="59" spans="3:9">
       <c r="F59" s="47"/>
       <c r="G59" s="47"/>
       <c r="H59" s="47"/>
       <c r="I59" s="47"/>
     </row>
-    <row r="60" spans="3:9" x14ac:dyDescent="0.2">
+    <row r="60" spans="3:9">
       <c r="F60" s="47"/>
       <c r="G60" s="47"/>
       <c r="H60" s="47"/>
       <c r="I60" s="47"/>
     </row>
-    <row r="61" spans="3:9" x14ac:dyDescent="0.2">
+    <row r="61" spans="3:9">
       <c r="F61" s="47"/>
       <c r="G61" s="47"/>
       <c r="H61" s="47"/>
       <c r="I61" s="47"/>
     </row>
-    <row r="62" spans="3:9" x14ac:dyDescent="0.2">
+    <row r="62" spans="3:9">
       <c r="F62" s="47"/>
       <c r="G62" s="47"/>
       <c r="H62" s="47"/>
       <c r="I62" s="47"/>
     </row>
-    <row r="63" spans="3:9" x14ac:dyDescent="0.2">
+    <row r="63" spans="3:9">
       <c r="F63" s="47"/>
       <c r="G63" s="47"/>
       <c r="H63" s="47"/>
       <c r="I63" s="47"/>
     </row>
-    <row r="64" spans="3:9" x14ac:dyDescent="0.2">
+    <row r="64" spans="3:9">
       <c r="F64" s="47"/>
       <c r="G64" s="47"/>
       <c r="H64" s="47"/>
       <c r="I64" s="47"/>
     </row>
-    <row r="65" spans="6:9" x14ac:dyDescent="0.2">
+    <row r="65" spans="6:9">
       <c r="F65" s="47"/>
       <c r="G65" s="47"/>
       <c r="H65" s="47"/>
       <c r="I65" s="47"/>
     </row>
-    <row r="66" spans="6:9" x14ac:dyDescent="0.2">
+    <row r="66" spans="6:9">
       <c r="F66" s="47"/>
       <c r="G66" s="47"/>
       <c r="H66" s="47"/>
       <c r="I66" s="47"/>
     </row>
-    <row r="67" spans="6:9" x14ac:dyDescent="0.2">
+    <row r="67" spans="6:9">
       <c r="F67" s="47"/>
       <c r="G67" s="47"/>
       <c r="H67" s="47"/>
       <c r="I67" s="47"/>
     </row>
-    <row r="68" spans="6:9" x14ac:dyDescent="0.2">
+    <row r="68" spans="6:9">
       <c r="F68" s="47"/>
       <c r="G68" s="47"/>
       <c r="H68" s="47"/>
       <c r="I68" s="47"/>
     </row>
-    <row r="69" spans="6:9" x14ac:dyDescent="0.2">
+    <row r="69" spans="6:9">
       <c r="F69" s="47"/>
       <c r="G69" s="47"/>
       <c r="H69" s="47"/>
       <c r="I69" s="47"/>
     </row>
-    <row r="70" spans="6:9" x14ac:dyDescent="0.2">
+    <row r="70" spans="6:9">
       <c r="F70" s="47"/>
       <c r="G70" s="47"/>
       <c r="H70" s="47"/>
       <c r="I70" s="47"/>
     </row>
-    <row r="71" spans="6:9" x14ac:dyDescent="0.2">
+    <row r="71" spans="6:9">
       <c r="F71" s="47"/>
       <c r="G71" s="47"/>
       <c r="H71" s="47"/>
       <c r="I71" s="47"/>
     </row>
-    <row r="72" spans="6:9" x14ac:dyDescent="0.2">
+    <row r="72" spans="6:9">
       <c r="F72" s="47"/>
       <c r="G72" s="47"/>
       <c r="H72" s="47"/>
       <c r="I72" s="47"/>
     </row>
-    <row r="73" spans="6:9" x14ac:dyDescent="0.2">
+    <row r="73" spans="6:9">
       <c r="F73" s="47"/>
       <c r="G73" s="47"/>
       <c r="H73" s="47"/>
       <c r="I73" s="47"/>
     </row>
-    <row r="74" spans="6:9" x14ac:dyDescent="0.2">
+    <row r="74" spans="6:9">
       <c r="F74" s="47"/>
       <c r="G74" s="47"/>
       <c r="H74" s="47"/>
       <c r="I74" s="47"/>
     </row>
-    <row r="75" spans="6:9" x14ac:dyDescent="0.2">
+    <row r="75" spans="6:9">
       <c r="F75" s="47"/>
       <c r="G75" s="47"/>
       <c r="H75" s="47"/>
       <c r="I75" s="47"/>
     </row>
-    <row r="76" spans="6:9" x14ac:dyDescent="0.2">
+    <row r="76" spans="6:9">
       <c r="F76" s="47"/>
       <c r="G76" s="47"/>
       <c r="H76" s="47"/>
       <c r="I76" s="47"/>
     </row>
-    <row r="77" spans="6:9" x14ac:dyDescent="0.2">
+    <row r="77" spans="6:9">
       <c r="F77" s="47"/>
       <c r="G77" s="47"/>
       <c r="H77" s="47"/>
       <c r="I77" s="47"/>
     </row>
-    <row r="78" spans="6:9" x14ac:dyDescent="0.2">
+    <row r="78" spans="6:9">
       <c r="F78" s="47"/>
       <c r="G78" s="47"/>
       <c r="H78" s="47"/>
       <c r="I78" s="47"/>
     </row>
-    <row r="79" spans="6:9" x14ac:dyDescent="0.2">
+    <row r="79" spans="6:9">
       <c r="F79" s="47"/>
       <c r="G79" s="47"/>
       <c r="H79" s="47"/>
       <c r="I79" s="47"/>
     </row>
-    <row r="80" spans="6:9" x14ac:dyDescent="0.2">
+    <row r="80" spans="6:9">
       <c r="F80" s="47"/>
       <c r="G80" s="47"/>
       <c r="H80" s="47"/>
       <c r="I80" s="47"/>
     </row>
-    <row r="81" spans="6:9" x14ac:dyDescent="0.2">
+    <row r="81" spans="6:9">
       <c r="F81" s="47"/>
       <c r="G81" s="47"/>
       <c r="H81" s="47"/>
       <c r="I81" s="47"/>
     </row>
-    <row r="82" spans="6:9" x14ac:dyDescent="0.2">
+    <row r="82" spans="6:9">
       <c r="F82" s="47"/>
       <c r="G82" s="47"/>
       <c r="H82" s="47"/>

</xml_diff>